<commit_message>
Publish Latest checklists 2026-09-18
Updates based on OWASP/wstg@8b3011c
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -2120,107 +2120,111 @@
       </c>
       <c r="F30" s="18" t="n"/>
     </row>
-    <row r="31" ht="15" customHeight="1" s="82">
-      <c r="A31" s="97" t="n"/>
-      <c r="B31" s="98" t="n"/>
-      <c r="C31" s="99" t="n"/>
-      <c r="D31" s="99" t="n"/>
-      <c r="E31" s="99" t="n"/>
-      <c r="F31" s="99" t="n"/>
-    </row>
-    <row r="32" ht="47.25" customHeight="1" s="82">
-      <c r="A32" s="9" t="n"/>
-      <c r="B32" s="100" t="inlineStr">
+    <row r="31" ht="247.5" customHeight="1" s="82">
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CONF-15</t>
+        </is>
+      </c>
+      <c r="C31" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/15-Feature_Flag_Security_Bypass", "Feature Flag Security Bypass")</f>
+        <v/>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>- Identify feature flags and kill-switches that control security-relevant functionality.
+- Determine whether feature flag states can be manipulated by an unauthorized client, and verify that backend security controls remain enforced independently of client-side flag state.
+- Verify that security controls remain consistently enforced across flag transitions, rollbacks, staged deployments, and services or instances, including whether stale security assertions or session state can be reused after a transition.
+- Evaluate fail-safe behavior when the feature flag service is unavailable.
+- Identify sensitive information exposed through feature flag configurations, and stale flags that may expose deprecated or unpatched code paths.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="82">
+      <c r="A32" s="97" t="n"/>
+      <c r="B32" s="98" t="n"/>
+      <c r="C32" s="99" t="n"/>
+      <c r="D32" s="99" t="n"/>
+      <c r="E32" s="99" t="n"/>
+      <c r="F32" s="99" t="n"/>
+    </row>
+    <row r="33" ht="47.25" customHeight="1" s="82">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="100" t="inlineStr">
         <is>
           <t>Identity Management</t>
         </is>
       </c>
-      <c r="C32" s="101" t="inlineStr">
+      <c r="C33" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D32" s="101" t="inlineStr">
+      <c r="D33" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E32" s="101" t="inlineStr">
+      <c r="E33" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F32" s="101" t="inlineStr">
+      <c r="F33" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="66" customHeight="1" s="82">
-      <c r="A33" s="19" t="n"/>
-      <c r="B33" s="34" t="inlineStr">
+    <row r="34" ht="66" customHeight="1" s="82">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-01</t>
         </is>
       </c>
-      <c r="C33" s="15">
+      <c r="C34" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/01-Role_Definitions", "Role Definitions")</f>
         <v/>
       </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>- Identify and document roles used by the application.
 - Attempt to switch, change, or access another role.
 - Review the granularity of the roles and the needs behind the permissions given.</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F33" s="18" t="n"/>
-    </row>
-    <row r="34" ht="49.5" customHeight="1" s="82">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="34" t="inlineStr">
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="n"/>
+    </row>
+    <row r="35" ht="49.5" customHeight="1" s="82">
+      <c r="A35" s="19" t="n"/>
+      <c r="B35" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-02</t>
         </is>
       </c>
-      <c r="C34" s="15">
+      <c r="C35" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/02-User_Registration_Process", "User Registration Process")</f>
         <v/>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>- Verify that the identity requirements for user registration are aligned with business and security requirements.
 - Validate the registration process.</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F34" s="18" t="n"/>
-    </row>
-    <row r="35" ht="33" customHeight="1" s="82">
-      <c r="A35" s="19" t="n"/>
-      <c r="B35" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-IDNT-03</t>
-        </is>
-      </c>
-      <c r="C35" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
-        <v/>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>- Verify which accounts may provision other accounts and of what type.</t>
-        </is>
-      </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2228,127 +2232,126 @@
       </c>
       <c r="F35" s="18" t="n"/>
     </row>
-    <row r="36" ht="49.5" customHeight="1" s="82">
+    <row r="36" ht="33" customHeight="1" s="82">
       <c r="A36" s="19" t="n"/>
       <c r="B36" s="34" t="inlineStr">
         <is>
+          <t>WSTG-IDNT-03</t>
+        </is>
+      </c>
+      <c r="C36" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
+        <v/>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>- Verify which accounts may provision other accounts and of what type.</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="n"/>
+    </row>
+    <row r="37" ht="49.5" customHeight="1" s="82">
+      <c r="A37" s="19" t="n"/>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
           <t>WSTG-IDNT-04</t>
         </is>
       </c>
-      <c r="C36" s="15">
+      <c r="C37" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/04-Account_Enumeration_and_Guessable_User_Account", "Account Enumeration and Guessable User Account")</f>
         <v/>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>- Review processes that pertain to user identification (*e.g.* registration, login, etc.).
 - Enumerate users where possible through response analysis.</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="n"/>
-    </row>
-    <row r="37" ht="16.5" customHeight="1" s="82">
-      <c r="A37" s="19" t="n"/>
-      <c r="B37" s="34" t="inlineStr">
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F37" s="18" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="82">
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-05</t>
         </is>
       </c>
-      <c r="C37" s="15">
+      <c r="C38" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/05-Weak_or_Unenforced_Username_Policy", "Weak or Unenforced Username Policy")</f>
         <v/>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E37" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F37" s="18" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="82">
-      <c r="A38" s="97" t="n"/>
-      <c r="B38" s="98" t="n"/>
-      <c r="C38" s="99" t="n"/>
-      <c r="D38" s="99" t="n"/>
-      <c r="E38" s="99" t="n"/>
-      <c r="F38" s="99" t="n"/>
-    </row>
-    <row r="39" ht="47.25" customHeight="1" s="82">
-      <c r="A39" s="9" t="n"/>
-      <c r="B39" s="100" t="inlineStr">
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F38" s="18" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="82">
+      <c r="A39" s="97" t="n"/>
+      <c r="B39" s="98" t="n"/>
+      <c r="C39" s="99" t="n"/>
+      <c r="D39" s="99" t="n"/>
+      <c r="E39" s="99" t="n"/>
+      <c r="F39" s="99" t="n"/>
+    </row>
+    <row r="40" ht="47.25" customHeight="1" s="82">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="100" t="inlineStr">
         <is>
           <t>Authentication</t>
         </is>
       </c>
-      <c r="C39" s="101" t="inlineStr">
+      <c r="C40" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D39" s="101" t="inlineStr">
+      <c r="D40" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E39" s="101" t="inlineStr">
+      <c r="E40" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F39" s="101" t="inlineStr">
+      <c r="F40" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="33" customHeight="1" s="82">
-      <c r="A40" s="19" t="n"/>
-      <c r="B40" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-01</t>
-        </is>
-      </c>
-      <c r="C40" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
-        <v/>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E40" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F40" s="18" t="n"/>
-    </row>
-    <row r="41" ht="66" customHeight="1" s="82">
+    <row r="41" ht="33" customHeight="1" s="82">
       <c r="A41" s="19" t="n"/>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-02</t>
+          <t>WSTG-ATHN-01</t>
         </is>
       </c>
       <c r="C41" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the application has any user accounts with default passwords.
-- Review whether new user accounts are created with weak or predictable passwords.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">
@@ -2362,40 +2365,41 @@
       <c r="A42" s="19" t="n"/>
       <c r="B42" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-02</t>
+        </is>
+      </c>
+      <c r="C42" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
+        <v/>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether the application has any user accounts with default passwords.
+- Review whether new user accounts are created with weak or predictable passwords.</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F42" s="18" t="n"/>
+    </row>
+    <row r="43" ht="66" customHeight="1" s="82">
+      <c r="A43" s="19" t="n"/>
+      <c r="B43" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-03</t>
         </is>
       </c>
-      <c r="C42" s="15">
+      <c r="C43" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/03-Weak_Lock_Out_Mechanism", "Weak Lock Out Mechanism")</f>
         <v/>
       </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>- Evaluate the account lockout mechanism's ability to mitigate brute force password guessing.
 - Evaluate the unlock mechanism's resistance to unauthorized account unlocking.</t>
-        </is>
-      </c>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F42" s="18" t="n"/>
-    </row>
-    <row r="43" ht="33" customHeight="1" s="82">
-      <c r="A43" s="19" t="n"/>
-      <c r="B43" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-04</t>
-        </is>
-      </c>
-      <c r="C43" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
-        <v/>
-      </c>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>- Ensure that authentication is applied across all services that require it.</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
@@ -2409,16 +2413,16 @@
       <c r="A44" s="19" t="n"/>
       <c r="B44" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-05</t>
+          <t>WSTG-ATHN-04</t>
         </is>
       </c>
       <c r="C44" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
+          <t>- Ensure that authentication is applied across all services that require it.</t>
         </is>
       </c>
       <c r="E44" s="18" t="inlineStr">
@@ -2428,46 +2432,46 @@
       </c>
       <c r="F44" s="18" t="n"/>
     </row>
-    <row r="45" ht="49.5" customHeight="1" s="82">
+    <row r="45" ht="33" customHeight="1" s="82">
       <c r="A45" s="19" t="n"/>
       <c r="B45" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-05</t>
+        </is>
+      </c>
+      <c r="C45" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
+        <v/>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F45" s="18" t="n"/>
+    </row>
+    <row r="46" ht="49.5" customHeight="1" s="82">
+      <c r="A46" s="19" t="n"/>
+      <c r="B46" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-06</t>
         </is>
       </c>
-      <c r="C45" s="15">
+      <c r="C46" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/06-Browser_Cache_Weaknesses", "Browser Cache Weaknesses")</f>
         <v/>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>- Review if the application stores sensitive information on the client-side.
 - Review if access can occur without authorization.</t>
         </is>
       </c>
-      <c r="E45" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F45" s="18" t="n"/>
-    </row>
-    <row r="46" ht="66" customHeight="1" s="82">
-      <c r="A46" s="19" t="n"/>
-      <c r="B46" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-07</t>
-        </is>
-      </c>
-      <c r="C46" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
-        <v/>
-      </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
-        </is>
-      </c>
       <c r="E46" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2475,46 +2479,46 @@
       </c>
       <c r="F46" s="18" t="n"/>
     </row>
-    <row r="47" ht="49.5" customHeight="1" s="82">
+    <row r="47" ht="66" customHeight="1" s="82">
       <c r="A47" s="19" t="n"/>
       <c r="B47" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-07</t>
+        </is>
+      </c>
+      <c r="C47" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
+        <v/>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
+        </is>
+      </c>
+      <c r="E47" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F47" s="18" t="n"/>
+    </row>
+    <row r="48" ht="49.5" customHeight="1" s="82">
+      <c r="A48" s="19" t="n"/>
+      <c r="B48" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-08</t>
         </is>
       </c>
-      <c r="C47" s="15">
+      <c r="C48" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/08-Weak_Security_Question_Answer", "Weak Security Question Answer")</f>
         <v/>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>- Determine the complexity and how straight-forward the questions are.
 - Assess possible user answers and brute force capabilities.</t>
         </is>
       </c>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F47" s="18" t="n"/>
-    </row>
-    <row r="48" ht="33" customHeight="1" s="82">
-      <c r="A48" s="19" t="n"/>
-      <c r="B48" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-09</t>
-        </is>
-      </c>
-      <c r="C48" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
-        <v/>
-      </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
-        </is>
-      </c>
       <c r="E48" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2522,131 +2526,131 @@
       </c>
       <c r="F48" s="18" t="n"/>
     </row>
-    <row r="49" ht="49.5" customHeight="1" s="82">
+    <row r="49" ht="33" customHeight="1" s="82">
       <c r="A49" s="19" t="n"/>
       <c r="B49" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-09</t>
+        </is>
+      </c>
+      <c r="C49" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
+        <v/>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F49" s="18" t="n"/>
+    </row>
+    <row r="50" ht="49.5" customHeight="1" s="82">
+      <c r="A50" s="19" t="n"/>
+      <c r="B50" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-10</t>
         </is>
       </c>
-      <c r="C49" s="15">
+      <c r="C50" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/10-Weaker_Authentication_in_Alternative_Channel", "Weaker Authentication in Alternative Channel")</f>
         <v/>
       </c>
-      <c r="D49" s="16" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>- Identify alternative authentication channels.
 - Assess the security measures used and if any bypasses exists on the alternative channels.</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F49" s="18" t="n"/>
-    </row>
-    <row r="50" ht="66" customHeight="1" s="82">
-      <c r="A50" s="19" t="n"/>
-      <c r="B50" s="34" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="n"/>
+    </row>
+    <row r="51" ht="66" customHeight="1" s="82">
+      <c r="A51" s="19" t="n"/>
+      <c r="B51" s="34" t="inlineStr">
         <is>
           <t>WSTG-ATHN-11</t>
         </is>
       </c>
-      <c r="C50" s="15">
+      <c r="C51" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/11-Multi-Factor_Authentication", "Multi-Factor Authentication (MFA)")</f>
         <v/>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>- Identify the type of MFA used by the application.
 - Determine whether the MFA implementation is robust and secure.
 - Attempt to bypass the MFA.</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="82">
-      <c r="A51" s="97" t="n"/>
-      <c r="B51" s="98" t="n"/>
-      <c r="C51" s="99" t="n"/>
-      <c r="D51" s="99" t="n"/>
-      <c r="E51" s="99" t="n"/>
-      <c r="F51" s="99" t="n"/>
-    </row>
-    <row r="52" ht="47.25" customHeight="1" s="82">
-      <c r="A52" s="9" t="n"/>
-      <c r="B52" s="100" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="n"/>
+    </row>
+    <row r="52" ht="15" customHeight="1" s="82">
+      <c r="A52" s="97" t="n"/>
+      <c r="B52" s="98" t="n"/>
+      <c r="C52" s="99" t="n"/>
+      <c r="D52" s="99" t="n"/>
+      <c r="E52" s="99" t="n"/>
+      <c r="F52" s="99" t="n"/>
+    </row>
+    <row r="53" ht="47.25" customHeight="1" s="82">
+      <c r="A53" s="9" t="n"/>
+      <c r="B53" s="100" t="inlineStr">
         <is>
           <t>Authorization</t>
         </is>
       </c>
-      <c r="C52" s="101" t="inlineStr">
+      <c r="C53" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D52" s="101" t="inlineStr">
+      <c r="D53" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E52" s="101" t="inlineStr">
+      <c r="E53" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F52" s="101" t="inlineStr">
+      <c r="F53" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="49.5" customHeight="1" s="82">
-      <c r="A53" s="19" t="n"/>
-      <c r="B53" s="34" t="inlineStr">
+    <row r="54" ht="49.5" customHeight="1" s="82">
+      <c r="A54" s="19" t="n"/>
+      <c r="B54" s="34" t="inlineStr">
         <is>
           <t>WSTG-ATHZ-01</t>
         </is>
       </c>
-      <c r="C53" s="15">
+      <c r="C54" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/01-Directory_Traversal_File_Include", "Directory Traversal File Include")</f>
         <v/>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>- Identify injection points that pertain to path traversal.
 - Assess bypassing techniques and identify the extent of path traversal.</t>
         </is>
       </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F53" s="18" t="n"/>
-    </row>
-    <row r="54" ht="33" customHeight="1" s="82">
-      <c r="A54" s="19" t="n"/>
-      <c r="B54" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHZ-02</t>
-        </is>
-      </c>
-      <c r="C54" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
-        <v/>
-      </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
-        </is>
-      </c>
       <c r="E54" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2654,21 +2658,20 @@
       </c>
       <c r="F54" s="18" t="n"/>
     </row>
-    <row r="55" ht="49.5" customHeight="1" s="82">
+    <row r="55" ht="33" customHeight="1" s="82">
       <c r="A55" s="19" t="n"/>
       <c r="B55" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-03</t>
+          <t>WSTG-ATHZ-02</t>
         </is>
       </c>
       <c r="C55" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points related to privilege manipulation.
-- Fuzz or otherwise attempt to bypass security measures.</t>
+          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
         </is>
       </c>
       <c r="E55" s="18" t="inlineStr">
@@ -2682,126 +2685,127 @@
       <c r="A56" s="19" t="n"/>
       <c r="B56" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHZ-03</t>
+        </is>
+      </c>
+      <c r="C56" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
+        <v/>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>- Identify injection points related to privilege manipulation.
+- Fuzz or otherwise attempt to bypass security measures.</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="n"/>
+    </row>
+    <row r="57" ht="49.5" customHeight="1" s="82">
+      <c r="A57" s="19" t="n"/>
+      <c r="B57" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHZ-04</t>
         </is>
       </c>
-      <c r="C56" s="15">
+      <c r="C57" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/04-Insecure_Direct_Object_References", "Insecure Direct Object References")</f>
         <v/>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>- Identify points where object references may occur.
 - Assess the access control measures and if they're vulnerable to IDOR.</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="n"/>
-    </row>
-    <row r="57" ht="33" customHeight="1" s="82">
-      <c r="A57" s="19" t="n"/>
-      <c r="B57" s="34" t="inlineStr">
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="n"/>
+    </row>
+    <row r="58" ht="33" customHeight="1" s="82">
+      <c r="A58" s="19" t="n"/>
+      <c r="B58" s="34" t="inlineStr">
         <is>
           <t>WSTG-ATHZ-05</t>
         </is>
       </c>
-      <c r="C57" s="15">
+      <c r="C58" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/05-OAuth_Weaknesses", "OAuth Weaknesses")</f>
         <v/>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>- Determine if OAuth2 implementation is vulnerable or using a deprecated or custom implementation.</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F57" s="18" t="n"/>
-    </row>
-    <row r="58" ht="15" customHeight="1" s="82">
-      <c r="A58" s="97" t="n"/>
-      <c r="B58" s="98" t="n"/>
-      <c r="C58" s="99" t="n"/>
-      <c r="D58" s="99" t="n"/>
-      <c r="E58" s="99" t="n"/>
-      <c r="F58" s="99" t="n"/>
-    </row>
-    <row r="59" ht="47.25" customHeight="1" s="82">
-      <c r="A59" s="9" t="n"/>
-      <c r="B59" s="100" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="n"/>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="82">
+      <c r="A59" s="97" t="n"/>
+      <c r="B59" s="98" t="n"/>
+      <c r="C59" s="99" t="n"/>
+      <c r="D59" s="99" t="n"/>
+      <c r="E59" s="99" t="n"/>
+      <c r="F59" s="99" t="n"/>
+    </row>
+    <row r="60" ht="47.25" customHeight="1" s="82">
+      <c r="A60" s="9" t="n"/>
+      <c r="B60" s="100" t="inlineStr">
         <is>
           <t>Session Management</t>
         </is>
       </c>
-      <c r="C59" s="101" t="inlineStr">
+      <c r="C60" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D59" s="101" t="inlineStr">
+      <c r="D60" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E59" s="101" t="inlineStr">
+      <c r="E60" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F59" s="101" t="inlineStr">
+      <c r="F60" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="99" customHeight="1" s="82">
-      <c r="A60" s="19" t="n"/>
-      <c r="B60" s="34" t="inlineStr">
+    <row r="61" ht="99" customHeight="1" s="82">
+      <c r="A61" s="19" t="n"/>
+      <c r="B61" s="34" t="inlineStr">
         <is>
           <t>WSTG-SESS-01</t>
         </is>
       </c>
-      <c r="C60" s="15">
+      <c r="C61" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/01-Session_Management_Schema", "Session Management Schema")</f>
         <v/>
       </c>
-      <c r="D60" s="16" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
         <is>
           <t>- Gather session tokens, for the same user and for different users where possible.
 - Analyze and ensure that enough randomness exists to stop session forging attacks.
 - Modify cookies that are not signed and contain information that can be manipulated.</t>
         </is>
       </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="n"/>
-    </row>
-    <row r="61" ht="33" customHeight="1" s="82">
-      <c r="A61" s="19" t="n"/>
-      <c r="B61" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-02</t>
-        </is>
-      </c>
-      <c r="C61" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
-        <v/>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>- Ensure that the proper security configuration is set for cookies.</t>
-        </is>
-      </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2813,67 +2817,67 @@
       <c r="A62" s="19" t="n"/>
       <c r="B62" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-02</t>
+        </is>
+      </c>
+      <c r="C62" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
+        <v/>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>- Ensure that the proper security configuration is set for cookies.</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="n"/>
+    </row>
+    <row r="63" ht="33" customHeight="1" s="82">
+      <c r="A63" s="19" t="n"/>
+      <c r="B63" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-03</t>
         </is>
       </c>
-      <c r="C62" s="15">
+      <c r="C63" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/03-Session_Fixation", "Session Fixation")</f>
         <v/>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>- Analyze the authentication mechanism and its flow.
 - Force cookies and assess the impact.</t>
         </is>
       </c>
-      <c r="E62" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F62" s="18" t="n"/>
-    </row>
-    <row r="63" ht="49.5" customHeight="1" s="82">
-      <c r="A63" s="19" t="n"/>
-      <c r="B63" s="34" t="inlineStr">
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="n"/>
+    </row>
+    <row r="64" ht="49.5" customHeight="1" s="82">
+      <c r="A64" s="19" t="n"/>
+      <c r="B64" s="34" t="inlineStr">
         <is>
           <t>WSTG-SESS-04</t>
         </is>
       </c>
-      <c r="C63" s="15">
+      <c r="C64" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/04-Exposed_Session_Variables", "Exposed Session Variables")</f>
         <v/>
       </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>- Ensure that proper encryption is implemented.
 - Review the caching configuration.
 - Assess the channel and methods' security.</t>
         </is>
       </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F63" s="18" t="n"/>
-    </row>
-    <row r="64" ht="33" customHeight="1" s="82">
-      <c r="A64" s="19" t="n"/>
-      <c r="B64" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-05</t>
-        </is>
-      </c>
-      <c r="C64" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
-        <v/>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
-        </is>
-      </c>
       <c r="E64" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2881,46 +2885,46 @@
       </c>
       <c r="F64" s="18" t="n"/>
     </row>
-    <row r="65" ht="49.5" customHeight="1" s="82">
+    <row r="65" ht="33" customHeight="1" s="82">
       <c r="A65" s="19" t="n"/>
       <c r="B65" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-05</t>
+        </is>
+      </c>
+      <c r="C65" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
+        <v/>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="n"/>
+    </row>
+    <row r="66" ht="49.5" customHeight="1" s="82">
+      <c r="A66" s="19" t="n"/>
+      <c r="B66" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-06</t>
         </is>
       </c>
-      <c r="C65" s="15">
+      <c r="C66" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/06-Logout_Functionality", "Logout Functionality")</f>
         <v/>
       </c>
-      <c r="D65" s="16" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
         <is>
           <t>- Assess the logout UI.
 - Analyze the session timeout and if the session is properly killed after logout.</t>
         </is>
       </c>
-      <c r="E65" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F65" s="18" t="n"/>
-    </row>
-    <row r="66" ht="16.5" customHeight="1" s="82">
-      <c r="A66" s="19" t="n"/>
-      <c r="B66" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-07</t>
-        </is>
-      </c>
-      <c r="C66" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
-        <v/>
-      </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>- Validate that a hard session timeout exists.</t>
-        </is>
-      </c>
       <c r="E66" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2928,21 +2932,20 @@
       </c>
       <c r="F66" s="18" t="n"/>
     </row>
-    <row r="67" ht="33" customHeight="1" s="82">
+    <row r="67" ht="16.5" customHeight="1" s="82">
       <c r="A67" s="19" t="n"/>
       <c r="B67" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-08</t>
+          <t>WSTG-SESS-07</t>
         </is>
       </c>
       <c r="C67" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
         <v/>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>- Identify all session variables.
-- Break the logical flow of session generation.</t>
+          <t>- Validate that a hard session timeout exists.</t>
         </is>
       </c>
       <c r="E67" s="18" t="inlineStr">
@@ -2956,41 +2959,41 @@
       <c r="A68" s="19" t="n"/>
       <c r="B68" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-08</t>
+        </is>
+      </c>
+      <c r="C68" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
+        <v/>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>- Identify all session variables.
+- Break the logical flow of session generation.</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="n"/>
+    </row>
+    <row r="69" ht="33" customHeight="1" s="82">
+      <c r="A69" s="19" t="n"/>
+      <c r="B69" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-09</t>
         </is>
       </c>
-      <c r="C68" s="15">
+      <c r="C69" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/09-Session_Hijacking", "Session Hijacking")</f>
         <v/>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
         <is>
           <t>- Identify vulnerable session cookies.
 - Hijack vulnerable cookies and assess the risk level.</t>
-        </is>
-      </c>
-      <c r="E68" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F68" s="18" t="n"/>
-    </row>
-    <row r="69" ht="49.5" customHeight="1" s="82">
-      <c r="A69" s="19" t="n"/>
-      <c r="B69" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-10</t>
-        </is>
-      </c>
-      <c r="C69" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
-        <v/>
-      </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>- Determine whether the JWTs expose sensitive information.
-- Determine whether the JWTs can be tampered with or modified.</t>
         </is>
       </c>
       <c r="E69" s="18" t="inlineStr">
@@ -3004,125 +3007,126 @@
       <c r="A70" s="19" t="n"/>
       <c r="B70" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-10</t>
+        </is>
+      </c>
+      <c r="C70" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
+        <v/>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether the JWTs expose sensitive information.
+- Determine whether the JWTs can be tampered with or modified.</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="n"/>
+    </row>
+    <row r="71" ht="49.5" customHeight="1" s="82">
+      <c r="A71" s="19" t="n"/>
+      <c r="B71" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-11</t>
         </is>
       </c>
-      <c r="C70" s="15">
+      <c r="C71" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/11-Concurrent_Sessions", "Concurrent Sessions")</f>
         <v/>
       </c>
-      <c r="D70" s="16" t="inlineStr">
+      <c r="D71" s="16" t="inlineStr">
         <is>
           <t>- Evaluate the application's session management by assessing the handling of multiple active sessions for a single user account.</t>
         </is>
       </c>
-      <c r="E70" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F70" s="18" t="n"/>
-    </row>
-    <row r="71" ht="15" customHeight="1" s="82">
-      <c r="A71" s="97" t="n"/>
-      <c r="B71" s="98" t="n"/>
-      <c r="C71" s="99" t="n"/>
-      <c r="D71" s="99" t="n"/>
-      <c r="E71" s="99" t="n"/>
-      <c r="F71" s="99" t="n"/>
-    </row>
-    <row r="72" ht="47.25" customHeight="1" s="82">
-      <c r="A72" s="9" t="n"/>
-      <c r="B72" s="100" t="inlineStr">
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="n"/>
+    </row>
+    <row r="72" ht="15" customHeight="1" s="82">
+      <c r="A72" s="97" t="n"/>
+      <c r="B72" s="98" t="n"/>
+      <c r="C72" s="99" t="n"/>
+      <c r="D72" s="99" t="n"/>
+      <c r="E72" s="99" t="n"/>
+      <c r="F72" s="99" t="n"/>
+    </row>
+    <row r="73" ht="47.25" customHeight="1" s="82">
+      <c r="A73" s="9" t="n"/>
+      <c r="B73" s="100" t="inlineStr">
         <is>
           <t>Injection</t>
         </is>
       </c>
-      <c r="C72" s="101" t="inlineStr">
+      <c r="C73" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D72" s="101" t="inlineStr">
+      <c r="D73" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E72" s="101" t="inlineStr">
+      <c r="E73" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F72" s="101" t="inlineStr">
+      <c r="F73" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="49.5" customHeight="1" s="82">
-      <c r="A73" s="19" t="n"/>
-      <c r="B73" s="34" t="inlineStr">
+    <row r="74" ht="49.5" customHeight="1" s="82">
+      <c r="A74" s="19" t="n"/>
+      <c r="B74" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-01</t>
         </is>
       </c>
-      <c r="C73" s="15">
+      <c r="C74" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/01-Reflected_Cross_Site_Scripting", "Reflected Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D73" s="16" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
         <is>
           <t>- Identify variables that are reflected in responses.
 - Assess the input they accept and the encoding that gets applied on return (if any).</t>
         </is>
       </c>
-      <c r="E73" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F73" s="18" t="n"/>
-    </row>
-    <row r="74" ht="66" customHeight="1" s="82">
-      <c r="A74" s="19" t="n"/>
-      <c r="B74" s="34" t="inlineStr">
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="n"/>
+    </row>
+    <row r="75" ht="66" customHeight="1" s="82">
+      <c r="A75" s="19" t="n"/>
+      <c r="B75" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-02</t>
         </is>
       </c>
-      <c r="C74" s="15">
+      <c r="C75" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/02-Stored_Cross_Site_Scripting", "Stored Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="D75" s="16" t="inlineStr">
         <is>
           <t>- Identify stored input that is reflected on the client-side.
 - Assess the input they accept and the encoding that gets applied on return (if any).</t>
         </is>
       </c>
-      <c r="E74" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F74" s="18" t="n"/>
-    </row>
-    <row r="75" ht="16.5" customHeight="1" s="82">
-      <c r="A75" s="19" t="n"/>
-      <c r="B75" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-03</t>
-        </is>
-      </c>
-      <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
-        <v/>
-      </c>
-      <c r="D75" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E75" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3130,21 +3134,20 @@
       </c>
       <c r="F75" s="18" t="n"/>
     </row>
-    <row r="76" ht="49.5" customHeight="1" s="82">
+    <row r="76" ht="16.5" customHeight="1" s="82">
       <c r="A76" s="19" t="n"/>
       <c r="B76" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INJT-04</t>
+          <t>WSTG-INJT-03</t>
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>- Identify the back end and the parsing method used.
-- Assess injection points and try bypassing input filters using HPP.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E76" s="18" t="inlineStr">
@@ -3158,114 +3161,115 @@
       <c r="A77" s="19" t="n"/>
       <c r="B77" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-04</t>
+        </is>
+      </c>
+      <c r="C77" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
+        <v/>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the back end and the parsing method used.
+- Assess injection points and try bypassing input filters using HPP.</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="n"/>
+    </row>
+    <row r="78" ht="49.5" customHeight="1" s="82">
+      <c r="A78" s="19" t="n"/>
+      <c r="B78" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-05</t>
         </is>
       </c>
-      <c r="C77" s="15">
+      <c r="C78" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/05-SQL_Injection", "SQL Injection")</f>
         <v/>
       </c>
-      <c r="D77" s="16" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>- Identify SQL injection points.
 - Assess the severity of the injection and the level of access that can be achieved through it.</t>
         </is>
       </c>
-      <c r="E77" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F77" s="18" t="n"/>
-    </row>
-    <row r="78" ht="33" customHeight="1" s="82">
-      <c r="A78" s="19" t="n"/>
-      <c r="B78" s="34" t="inlineStr">
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="n"/>
+    </row>
+    <row r="79" ht="33" customHeight="1" s="82">
+      <c r="A79" s="19" t="n"/>
+      <c r="B79" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-06</t>
         </is>
       </c>
-      <c r="C78" s="15">
+      <c r="C79" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/06-LDAP_Injection", "LDAP Injection")</f>
         <v/>
       </c>
-      <c r="D78" s="16" t="inlineStr">
+      <c r="D79" s="16" t="inlineStr">
         <is>
           <t>- Identify LDAP injection points.
 - Assess the severity of the injection.</t>
         </is>
       </c>
-      <c r="E78" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F78" s="18" t="n"/>
-    </row>
-    <row r="79" ht="49.5" customHeight="1" s="82">
-      <c r="A79" s="19" t="n"/>
-      <c r="B79" s="34" t="inlineStr">
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="n"/>
+    </row>
+    <row r="80" ht="49.5" customHeight="1" s="82">
+      <c r="A80" s="19" t="n"/>
+      <c r="B80" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-07</t>
         </is>
       </c>
-      <c r="C79" s="15">
+      <c r="C80" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/07-XML_Injection", "XML Injection")</f>
         <v/>
       </c>
-      <c r="D79" s="16" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>- Identify XML injection points.
 - Assess the types of exploits that can be attained and their severities.</t>
         </is>
       </c>
-      <c r="E79" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F79" s="18" t="n"/>
-    </row>
-    <row r="80" ht="33" customHeight="1" s="82">
-      <c r="A80" s="19" t="n"/>
-      <c r="B80" s="34" t="inlineStr">
+      <c r="E80" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="n"/>
+    </row>
+    <row r="81" ht="33" customHeight="1" s="82">
+      <c r="A81" s="19" t="n"/>
+      <c r="B81" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-08</t>
         </is>
       </c>
-      <c r="C80" s="15">
+      <c r="C81" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/08-SSI_Injection", "SSI Injection")</f>
         <v/>
       </c>
-      <c r="D80" s="16" t="inlineStr">
+      <c r="D81" s="16" t="inlineStr">
         <is>
           <t>- Identify SSI injection points.
 - Assess the severity of the injection.</t>
         </is>
       </c>
-      <c r="E80" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F80" s="18" t="n"/>
-    </row>
-    <row r="81" ht="16.5" customHeight="1" s="82">
-      <c r="A81" s="19" t="n"/>
-      <c r="B81" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-09</t>
-        </is>
-      </c>
-      <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
-        <v/>
-      </c>
-      <c r="D81" s="16" t="inlineStr">
-        <is>
-          <t>- Identify XPATH injection points.</t>
-        </is>
-      </c>
       <c r="E81" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3273,95 +3277,95 @@
       </c>
       <c r="F81" s="18" t="n"/>
     </row>
-    <row r="82" ht="66" customHeight="1" s="82">
+    <row r="82" ht="16.5" customHeight="1" s="82">
       <c r="A82" s="19" t="n"/>
       <c r="B82" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-09</t>
+        </is>
+      </c>
+      <c r="C82" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
+        <v/>
+      </c>
+      <c r="D82" s="16" t="inlineStr">
+        <is>
+          <t>- Identify XPATH injection points.</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="n"/>
+    </row>
+    <row r="83" ht="66" customHeight="1" s="82">
+      <c r="A83" s="19" t="n"/>
+      <c r="B83" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-10</t>
         </is>
       </c>
-      <c r="C82" s="15">
+      <c r="C83" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/10-IMAP_SMTP_Injection", "IMAP SMTP Injection")</f>
         <v/>
       </c>
-      <c r="D82" s="16" t="inlineStr">
+      <c r="D83" s="16" t="inlineStr">
         <is>
           <t>- Identify IMAP/SMTP injection points.
 - Understand the data flow and deployment structure of the system.
 - Assess the injection impacts.</t>
         </is>
       </c>
-      <c r="E82" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F82" s="18" t="n"/>
-    </row>
-    <row r="83" ht="49.5" customHeight="1" s="82">
-      <c r="A83" s="19" t="n"/>
-      <c r="B83" s="34" t="inlineStr">
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="n"/>
+    </row>
+    <row r="84" ht="49.5" customHeight="1" s="82">
+      <c r="A84" s="19" t="n"/>
+      <c r="B84" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-11</t>
         </is>
       </c>
-      <c r="C83" s="15">
+      <c r="C84" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/11-Code_Injection", "Code Injection")</f>
         <v/>
       </c>
-      <c r="D83" s="16" t="inlineStr">
+      <c r="D84" s="16" t="inlineStr">
         <is>
           <t>- Identify injection points where you can inject code into the application.
 - Assess the injection severity.</t>
         </is>
       </c>
-      <c r="E83" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F83" s="18" t="n"/>
-    </row>
-    <row r="84" ht="33" customHeight="1" s="82">
-      <c r="A84" s="19" t="n"/>
-      <c r="B84" s="34" t="inlineStr">
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="n"/>
+    </row>
+    <row r="85" ht="33" customHeight="1" s="82">
+      <c r="A85" s="19" t="n"/>
+      <c r="B85" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-12</t>
         </is>
       </c>
-      <c r="C84" s="15">
+      <c r="C85" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/12-Command_Injection", "Command Injection")</f>
         <v/>
       </c>
-      <c r="D84" s="16" t="inlineStr">
+      <c r="D85" s="16" t="inlineStr">
         <is>
           <t>- Identify and assess command injection points.
 - Bypass special characters and OS commands filter.</t>
         </is>
       </c>
-      <c r="E84" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F84" s="18" t="n"/>
-    </row>
-    <row r="85" ht="49.5" customHeight="1" s="82">
-      <c r="A85" s="19" t="n"/>
-      <c r="B85" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-13</t>
-        </is>
-      </c>
-      <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
-        <v/>
-      </c>
-      <c r="D85" s="16" t="inlineStr">
-        <is>
-          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
-        </is>
-      </c>
       <c r="E85" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3369,68 +3373,91 @@
       </c>
       <c r="F85" s="18" t="n"/>
     </row>
-    <row r="86" ht="66" customHeight="1" s="82">
+    <row r="86" ht="49.5" customHeight="1" s="82">
       <c r="A86" s="19" t="n"/>
       <c r="B86" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-13</t>
+        </is>
+      </c>
+      <c r="C86" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
+        <v/>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="n"/>
+    </row>
+    <row r="87" ht="66" customHeight="1" s="82">
+      <c r="A87" s="19" t="n"/>
+      <c r="B87" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-14</t>
         </is>
       </c>
-      <c r="C86" s="15">
+      <c r="C87" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/14-Incubated_Vulnerability", "Incubated Vulnerability")</f>
         <v/>
       </c>
-      <c r="D86" s="16" t="inlineStr">
+      <c r="D87" s="16" t="inlineStr">
         <is>
           <t>- Identify injections that are stored and require a recall step to the stored injection.
 - Understand how a recall step could occur.
 - Set listeners or activate the recall step if possible.</t>
         </is>
       </c>
-      <c r="E86" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F86" s="18" t="n"/>
-    </row>
-    <row r="87" ht="115.5" customHeight="1" s="82">
-      <c r="A87" s="19" t="n"/>
-      <c r="B87" s="34" t="inlineStr">
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="n"/>
+    </row>
+    <row r="88" ht="115.5" customHeight="1" s="82">
+      <c r="A88" s="19" t="n"/>
+      <c r="B88" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-15</t>
         </is>
       </c>
-      <c r="C87" s="15">
+      <c r="C88" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/15-HTTP_Response_Splitting", "HTTP Response Splitting")</f>
         <v/>
       </c>
-      <c r="D87" s="16" t="inlineStr">
+      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>- Identify user-controlled input that is reflected into HTTP response headers.
 - Assess whether CR (`\r`) and LF (`\n`) characters can be injected into response headers.
 - Determine the potential impact of successful HTTP Response Splitting attacks, such as cache poisoning or client-side exploitation.</t>
         </is>
       </c>
-      <c r="E87" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F87" s="18" t="n"/>
-    </row>
-    <row r="88" ht="99" customHeight="1" s="82">
-      <c r="A88" s="19" t="n"/>
-      <c r="B88" s="34" t="inlineStr">
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="n"/>
+    </row>
+    <row r="89" ht="99" customHeight="1" s="82">
+      <c r="A89" s="19" t="n"/>
+      <c r="B89" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-16</t>
         </is>
       </c>
-      <c r="C88" s="15">
+      <c r="C89" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/16-HTTP_Request_Smuggling", "HTTP Request Smuggling")</f>
         <v/>
       </c>
-      <c r="D88" s="16" t="inlineStr">
+      <c r="D89" s="16" t="inlineStr">
         <is>
           <t>- Identify request boundary inconsistencies between frontend and backend components
 - Detect classic CL/TE desynchronization vulnerabilities
@@ -3439,30 +3466,6 @@
 - Confirm backend request queue poisoning</t>
         </is>
       </c>
-      <c r="E88" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F88" s="18" t="n"/>
-    </row>
-    <row r="89" ht="49.5" customHeight="1" s="82">
-      <c r="A89" s="19" t="n"/>
-      <c r="B89" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-17</t>
-        </is>
-      </c>
-      <c r="C89" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
-        <v/>
-      </c>
-      <c r="D89" s="16" t="inlineStr">
-        <is>
-          <t>- Assess if the Host header is being parsed dynamically in the application.
-- Bypass security controls that rely on the header.</t>
-        </is>
-      </c>
       <c r="E89" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3474,88 +3477,112 @@
       <c r="A90" s="19" t="n"/>
       <c r="B90" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-17</t>
+        </is>
+      </c>
+      <c r="C90" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
+        <v/>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>- Assess if the Host header is being parsed dynamically in the application.
+- Bypass security controls that rely on the header.</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="n"/>
+    </row>
+    <row r="91" ht="49.5" customHeight="1" s="82">
+      <c r="A91" s="19" t="n"/>
+      <c r="B91" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-18</t>
         </is>
       </c>
-      <c r="C90" s="15">
+      <c r="C91" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/18-Server-side_Template_Injection", "Server-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="D91" s="16" t="inlineStr">
         <is>
           <t>- Detect template injection vulnerability points.
 - Identify the templating engine.
 - Build the exploit.</t>
         </is>
       </c>
-      <c r="E90" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F90" s="18" t="n"/>
-    </row>
-    <row r="91" ht="49.5" customHeight="1" s="82">
-      <c r="A91" s="19" t="n"/>
-      <c r="B91" s="34" t="inlineStr">
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="n"/>
+    </row>
+    <row r="92" ht="49.5" customHeight="1" s="82">
+      <c r="A92" s="19" t="n"/>
+      <c r="B92" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-19</t>
         </is>
       </c>
-      <c r="C91" s="15">
+      <c r="C92" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/19-Server-Side_Request_Forgery", "Server-Side Request Forgery")</f>
         <v/>
       </c>
-      <c r="D91" s="16" t="inlineStr">
+      <c r="D92" s="16" t="inlineStr">
         <is>
           <t>- Identify SSRF injection points.
 - Test if the injection points are exploitable.
 - Asses the severity of the vulnerability.</t>
         </is>
       </c>
-      <c r="E91" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F91" s="18" t="n"/>
-    </row>
-    <row r="92" ht="49.5" customHeight="1" s="82">
-      <c r="A92" s="19" t="n"/>
-      <c r="B92" s="34" t="inlineStr">
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="n"/>
+    </row>
+    <row r="93" ht="49.5" customHeight="1" s="82">
+      <c r="A93" s="19" t="n"/>
+      <c r="B93" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-20</t>
         </is>
       </c>
-      <c r="C92" s="15">
+      <c r="C93" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/20-Mass_Assignment", "Mass Assignment")</f>
         <v/>
       </c>
-      <c r="D92" s="16" t="inlineStr">
+      <c r="D93" s="16" t="inlineStr">
         <is>
           <t>- Identify requests that modify objects
 - Assess if it is possible to modify fields never intended to be modified from outside</t>
         </is>
       </c>
-      <c r="E92" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F92" s="18" t="n"/>
-    </row>
-    <row r="93" ht="181.5" customHeight="1" s="82">
-      <c r="A93" s="19" t="n"/>
-      <c r="B93" s="34" t="inlineStr">
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="n"/>
+    </row>
+    <row r="94" ht="181.5" customHeight="1" s="82">
+      <c r="A94" s="19" t="n"/>
+      <c r="B94" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-21</t>
         </is>
       </c>
-      <c r="C93" s="15">
+      <c r="C94" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/21-CSV_Injection", "CSV Injection")</f>
         <v/>
       </c>
-      <c r="D93" s="16" t="inlineStr">
+      <c r="D94" s="16" t="inlineStr">
         <is>
           <t>- Identify CSV/spreadsheet export features that include untrusted input.
 - Verify whether attacker-controlled values are interpreted as formulas when the export is opened in common spreadsheet applications.
@@ -3564,50 +3591,50 @@
 - Assess practical impact based on who opens the export and how it is used.</t>
         </is>
       </c>
-      <c r="E93" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F93" s="18" t="n"/>
-    </row>
-    <row r="94" ht="99" customHeight="1" s="82">
-      <c r="A94" s="19" t="n"/>
-      <c r="B94" s="34" t="inlineStr">
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="n"/>
+    </row>
+    <row r="95" ht="99" customHeight="1" s="82">
+      <c r="A95" s="19" t="n"/>
+      <c r="B95" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-22</t>
         </is>
       </c>
-      <c r="C94" s="15">
+      <c r="C95" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/22-Prototype_Pollution", "Prototype Pollution")</f>
         <v/>
       </c>
-      <c r="D94" s="16" t="inlineStr">
+      <c r="D95" s="16" t="inlineStr">
         <is>
           <t>- Identify functions and libraries that recursively merge, clone, or assign user-controlled properties.
 - Determine whether user input can reach and modify `Object.prototype`.
 - Identify gadgets that turn prototype pollution into a concrete impact.</t>
         </is>
       </c>
-      <c r="E94" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F94" s="18" t="n"/>
-    </row>
-    <row r="95" ht="165" customHeight="1" s="82">
-      <c r="A95" s="19" t="n"/>
-      <c r="B95" s="34" t="inlineStr">
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="n"/>
+    </row>
+    <row r="96" ht="165" customHeight="1" s="82">
+      <c r="A96" s="19" t="n"/>
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-23</t>
         </is>
       </c>
-      <c r="C95" s="15">
+      <c r="C96" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/23-Insecure_Deserialization", "Insecure Deserialization")</f>
         <v/>
       </c>
-      <c r="D95" s="16" t="inlineStr">
+      <c r="D96" s="16" t="inlineStr">
         <is>
           <t>- Identify entry points where the application accepts serialized objects from untrusted
 - urces (for example, HTTP headers, parameters, or cookies).
@@ -3617,174 +3644,150 @@
 - pact.</t>
         </is>
       </c>
-      <c r="E95" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F95" s="18" t="n"/>
-    </row>
-    <row r="96" ht="15" customHeight="1" s="82">
-      <c r="A96" s="97" t="n"/>
-      <c r="B96" s="98" t="n"/>
-      <c r="C96" s="99" t="n"/>
-      <c r="D96" s="99" t="n"/>
-      <c r="E96" s="99" t="n"/>
-      <c r="F96" s="99" t="n"/>
-    </row>
-    <row r="97" ht="47.25" customHeight="1" s="82">
-      <c r="A97" s="9" t="n"/>
-      <c r="B97" s="100" t="inlineStr">
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="n"/>
+    </row>
+    <row r="97" ht="15" customHeight="1" s="82">
+      <c r="A97" s="97" t="n"/>
+      <c r="B97" s="98" t="n"/>
+      <c r="C97" s="99" t="n"/>
+      <c r="D97" s="99" t="n"/>
+      <c r="E97" s="99" t="n"/>
+      <c r="F97" s="99" t="n"/>
+    </row>
+    <row r="98" ht="47.25" customHeight="1" s="82">
+      <c r="A98" s="9" t="n"/>
+      <c r="B98" s="100" t="inlineStr">
         <is>
           <t>Error Handling</t>
         </is>
       </c>
-      <c r="C97" s="101" t="inlineStr">
+      <c r="C98" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D97" s="101" t="inlineStr">
+      <c r="D98" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E97" s="101" t="inlineStr">
+      <c r="E98" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F97" s="101" t="inlineStr">
+      <c r="F98" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="33" customHeight="1" s="82">
-      <c r="A98" s="19" t="n"/>
-      <c r="B98" s="34" t="inlineStr">
+    <row r="99" ht="33" customHeight="1" s="82">
+      <c r="A99" s="19" t="n"/>
+      <c r="B99" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C98" s="15">
+      <c r="C99" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/01-Improper_Error_Handling", "Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D99" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="n"/>
-    </row>
-    <row r="99" ht="16.5" customHeight="1" s="82">
-      <c r="A99" s="19" t="n"/>
-      <c r="B99" s="34" t="inlineStr">
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="n"/>
+    </row>
+    <row r="100" ht="16.5" customHeight="1" s="82">
+      <c r="A100" s="19" t="n"/>
+      <c r="B100" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C99" s="15">
+      <c r="C100" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/02-Stack_Traces", "Stack Traces")</f>
         <v/>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D100" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E99" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F99" s="18" t="n"/>
-    </row>
-    <row r="100" ht="15" customHeight="1" s="82">
-      <c r="A100" s="97" t="n"/>
-      <c r="B100" s="98" t="n"/>
-      <c r="C100" s="99" t="n"/>
-      <c r="D100" s="99" t="n"/>
-      <c r="E100" s="99" t="n"/>
-      <c r="F100" s="99" t="n"/>
-    </row>
-    <row r="101" ht="47.25" customHeight="1" s="82">
-      <c r="A101" s="9" t="n"/>
-      <c r="B101" s="100" t="inlineStr">
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="n"/>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="82">
+      <c r="A101" s="97" t="n"/>
+      <c r="B101" s="98" t="n"/>
+      <c r="C101" s="99" t="n"/>
+      <c r="D101" s="99" t="n"/>
+      <c r="E101" s="99" t="n"/>
+      <c r="F101" s="99" t="n"/>
+    </row>
+    <row r="102" ht="47.25" customHeight="1" s="82">
+      <c r="A102" s="9" t="n"/>
+      <c r="B102" s="100" t="inlineStr">
         <is>
           <t>Weak Cryptography</t>
         </is>
       </c>
-      <c r="C101" s="101" t="inlineStr">
+      <c r="C102" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D101" s="101" t="inlineStr">
+      <c r="D102" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E101" s="101" t="inlineStr">
+      <c r="E102" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F101" s="101" t="inlineStr">
+      <c r="F102" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="82.5" customHeight="1" s="82">
-      <c r="A102" s="19" t="n"/>
-      <c r="B102" s="34" t="inlineStr">
+    <row r="103" ht="82.5" customHeight="1" s="82">
+      <c r="A103" s="19" t="n"/>
+      <c r="B103" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C102" s="15">
+      <c r="C103" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/01-Weak_Transport_Layer_Security", "Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D103" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
-      <c r="E102" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F102" s="18" t="n"/>
-    </row>
-    <row r="103" ht="49.5" customHeight="1" s="82">
-      <c r="A103" s="19" t="n"/>
-      <c r="B103" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-02</t>
-        </is>
-      </c>
-      <c r="C103" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
-        <v/>
-      </c>
-      <c r="D103" s="16" t="inlineStr">
-        <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
-        </is>
-      </c>
       <c r="E103" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3796,146 +3799,170 @@
       <c r="A104" s="19" t="n"/>
       <c r="B104" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C104" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="n"/>
+    </row>
+    <row r="105" ht="49.5" customHeight="1" s="82">
+      <c r="A105" s="19" t="n"/>
+      <c r="B105" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CRYP-03</t>
         </is>
       </c>
-      <c r="C104" s="15">
+      <c r="C105" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/03-Sensitive_Information_Sent_via_Unencrypted_Channels", "Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="D105" s="16" t="inlineStr">
         <is>
           <t>- Identify sensitive information transmitted through the various channels.
 - Assess the privacy and security of the channels used.</t>
         </is>
       </c>
-      <c r="E104" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F104" s="18" t="n"/>
-    </row>
-    <row r="105" ht="33" customHeight="1" s="82">
-      <c r="A105" s="19" t="n"/>
-      <c r="B105" s="34" t="inlineStr">
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="n"/>
+    </row>
+    <row r="106" ht="33" customHeight="1" s="82">
+      <c r="A106" s="19" t="n"/>
+      <c r="B106" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-04</t>
         </is>
       </c>
-      <c r="C105" s="15">
+      <c r="C106" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/04-Weak_Cryptographic_Primitives", "Weak Cryptographic Primitives")</f>
         <v/>
       </c>
-      <c r="D105" s="16" t="inlineStr">
+      <c r="D106" s="16" t="inlineStr">
         <is>
           <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
-      <c r="E105" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F105" s="18" t="n"/>
-    </row>
-    <row r="106" ht="15" customHeight="1" s="82">
-      <c r="A106" s="97" t="n"/>
-      <c r="B106" s="98" t="n"/>
-      <c r="C106" s="99" t="n"/>
-      <c r="D106" s="99" t="n"/>
-      <c r="E106" s="99" t="n"/>
-      <c r="F106" s="99" t="n"/>
-    </row>
-    <row r="107" ht="47.25" customHeight="1" s="82">
-      <c r="A107" s="9" t="n"/>
-      <c r="B107" s="100" t="inlineStr">
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="n"/>
+    </row>
+    <row r="107" ht="15" customHeight="1" s="82">
+      <c r="A107" s="97" t="n"/>
+      <c r="B107" s="98" t="n"/>
+      <c r="C107" s="99" t="n"/>
+      <c r="D107" s="99" t="n"/>
+      <c r="E107" s="99" t="n"/>
+      <c r="F107" s="99" t="n"/>
+    </row>
+    <row r="108" ht="47.25" customHeight="1" s="82">
+      <c r="A108" s="9" t="n"/>
+      <c r="B108" s="100" t="inlineStr">
         <is>
           <t>Business Logic</t>
         </is>
       </c>
-      <c r="C107" s="101" t="inlineStr">
+      <c r="C108" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D107" s="101" t="inlineStr">
+      <c r="D108" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E107" s="101" t="inlineStr">
+      <c r="E108" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F107" s="101" t="inlineStr">
+      <c r="F108" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="82.5" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+    <row r="109" ht="82.5" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C109" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/01-Business_Logic_Data_Validation", "Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="66" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="66" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C110" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/02-Ability_to_Forge_Requests", "Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="148.5" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="n"/>
+    </row>
+    <row r="111" ht="148.5" customHeight="1" s="82">
+      <c r="A111" s="19" t="n"/>
+      <c r="B111" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C111" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/03-Integrity_Checks", "Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D111" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3943,147 +3970,147 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F110" s="18" t="n"/>
-    </row>
-    <row r="111" ht="49.5" customHeight="1" s="82">
-      <c r="A111" s="19" t="n"/>
-      <c r="B111" s="34" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="n"/>
+    </row>
+    <row r="112" ht="49.5" customHeight="1" s="82">
+      <c r="A112" s="19" t="n"/>
+      <c r="B112" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-04</t>
         </is>
       </c>
-      <c r="C111" s="15">
+      <c r="C112" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/04-Process_Timing", "Process Timing")</f>
         <v/>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D112" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for system functionality that may be impacted by time.
 - Develop and execute misuse cases.</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F111" s="18" t="n"/>
-    </row>
-    <row r="112" ht="66" customHeight="1" s="82">
-      <c r="A112" s="19" t="n"/>
-      <c r="B112" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="66" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-05</t>
         </is>
       </c>
-      <c r="C112" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/05-Number_of_Times_a_Function_Can_Be_Used_Limits", "Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Identify functions that must set limits to the times they can be called.
 - Assess if there is a logical limit set on the functions and if it is properly validated.</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="82.5" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="82.5" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-06</t>
         </is>
       </c>
-      <c r="C113" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/06-Circumvention_of_Work_Flows", "Circumvention of Work Flows")</f>
         <v/>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
 - Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="99" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="99" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-07</t>
         </is>
       </c>
-      <c r="C114" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/07-Defenses_Against_Application_Misuse", "Defenses Against Application Misuse")</f>
         <v/>
       </c>
-      <c r="D114" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="99" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="99" customHeight="1" s="82">
+      <c r="A116" s="19" t="n"/>
+      <c r="B116" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C116" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/08-Upload_of_Unexpected_File_Types", "Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="165" customHeight="1" s="82">
-      <c r="A116" s="19" t="n"/>
-      <c r="B116" s="34" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="n"/>
+    </row>
+    <row r="117" ht="165" customHeight="1" s="82">
+      <c r="A117" s="19" t="n"/>
+      <c r="B117" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C116" s="15">
+      <c r="C117" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/09-Upload_of_Malicious_Files", "Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D116" s="16" t="inlineStr">
+      <c r="D117" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4093,114 +4120,91 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F116" s="18" t="n"/>
-    </row>
-    <row r="117" ht="66" customHeight="1" s="82">
-      <c r="A117" s="19" t="n"/>
-      <c r="B117" s="34" t="inlineStr">
+      <c r="E117" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F117" s="18" t="n"/>
+    </row>
+    <row r="118" ht="66" customHeight="1" s="82">
+      <c r="A118" s="19" t="n"/>
+      <c r="B118" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C117" s="15">
+      <c r="C118" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/10-Payment_Functionality", "Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D117" s="16" t="inlineStr">
+      <c r="D118" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E117" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F117" s="18" t="n"/>
-    </row>
-    <row r="118" ht="15" customHeight="1" s="82">
-      <c r="A118" s="97" t="n"/>
-      <c r="B118" s="98" t="n"/>
-      <c r="C118" s="99" t="n"/>
-      <c r="D118" s="99" t="n"/>
-      <c r="E118" s="99" t="n"/>
-      <c r="F118" s="99" t="n"/>
-    </row>
-    <row r="119" ht="47.25" customHeight="1" s="82">
-      <c r="A119" s="9" t="n"/>
-      <c r="B119" s="100" t="inlineStr">
+      <c r="E118" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="n"/>
+    </row>
+    <row r="119" ht="15" customHeight="1" s="82">
+      <c r="A119" s="97" t="n"/>
+      <c r="B119" s="98" t="n"/>
+      <c r="C119" s="99" t="n"/>
+      <c r="D119" s="99" t="n"/>
+      <c r="E119" s="99" t="n"/>
+      <c r="F119" s="99" t="n"/>
+    </row>
+    <row r="120" ht="47.25" customHeight="1" s="82">
+      <c r="A120" s="9" t="n"/>
+      <c r="B120" s="100" t="inlineStr">
         <is>
           <t>Client-side</t>
         </is>
       </c>
-      <c r="C119" s="101" t="inlineStr">
+      <c r="C120" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D119" s="101" t="inlineStr">
+      <c r="D120" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E119" s="101" t="inlineStr">
+      <c r="E120" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F119" s="101" t="inlineStr">
+      <c r="F120" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="33" customHeight="1" s="82">
-      <c r="A120" s="19" t="n"/>
-      <c r="B120" s="34" t="inlineStr">
+    <row r="121" ht="33" customHeight="1" s="82">
+      <c r="A121" s="19" t="n"/>
+      <c r="B121" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-01</t>
         </is>
       </c>
-      <c r="C120" s="15">
+      <c r="C121" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/01-DOM-based_Cross_Site_Scripting", "DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D120" s="16" t="inlineStr">
+      <c r="D121" s="16" t="inlineStr">
         <is>
           <t>- Identify DOM sinks.
 - Build payloads that pertain to every sink type.</t>
         </is>
       </c>
-      <c r="E120" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F120" s="18" t="n"/>
-    </row>
-    <row r="121" ht="16.5" customHeight="1" s="82">
-      <c r="A121" s="19" t="n"/>
-      <c r="B121" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-02</t>
-        </is>
-      </c>
-      <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
-        <v/>
-      </c>
-      <c r="D121" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
-        </is>
-      </c>
       <c r="E121" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4208,20 +4212,20 @@
       </c>
       <c r="F121" s="18" t="n"/>
     </row>
-    <row r="122" ht="33" customHeight="1" s="82">
+    <row r="122" ht="16.5" customHeight="1" s="82">
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-02</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4235,17 +4239,16 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4259,17 +4262,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4283,17 +4286,17 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C125" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
         <v/>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E125" s="18" t="inlineStr">
@@ -4307,42 +4310,43 @@
       <c r="A126" s="19" t="n"/>
       <c r="B126" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-06</t>
+        </is>
+      </c>
+      <c r="C126" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
+        <v/>
+      </c>
+      <c r="D126" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
+        </is>
+      </c>
+      <c r="E126" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F126" s="18" t="n"/>
+    </row>
+    <row r="127" ht="33" customHeight="1" s="82">
+      <c r="A127" s="19" t="n"/>
+      <c r="B127" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-07</t>
         </is>
       </c>
-      <c r="C126" s="15">
+      <c r="C127" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/07-Cross_Origin_Resource_Sharing", "Cross Origin Resource Sharing")</f>
         <v/>
       </c>
-      <c r="D126" s="16" t="inlineStr">
+      <c r="D127" s="16" t="inlineStr">
         <is>
           <t>- Identify endpoints that implement CORS.
 - Ensure that the CORS configuration is secure or harmless.</t>
         </is>
       </c>
-      <c r="E126" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F126" s="18" t="n"/>
-    </row>
-    <row r="127" ht="16.5" customHeight="1" s="82">
-      <c r="A127" s="19" t="n"/>
-      <c r="B127" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-09</t>
-        </is>
-      </c>
-      <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
-        <v/>
-      </c>
-      <c r="D127" s="16" t="inlineStr">
-        <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
-        </is>
-      </c>
       <c r="E127" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4350,21 +4354,20 @@
       </c>
       <c r="F127" s="18" t="n"/>
     </row>
-    <row r="128" ht="49.5" customHeight="1" s="82">
+    <row r="128" ht="16.5" customHeight="1" s="82">
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E128" s="18" t="inlineStr">
@@ -4378,90 +4381,91 @@
       <c r="A129" s="19" t="n"/>
       <c r="B129" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-10</t>
+        </is>
+      </c>
+      <c r="C129" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
+        <v/>
+      </c>
+      <c r="D129" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
+        </is>
+      </c>
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="n"/>
+    </row>
+    <row r="130" ht="49.5" customHeight="1" s="82">
+      <c r="A130" s="19" t="n"/>
+      <c r="B130" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-11</t>
         </is>
       </c>
-      <c r="C129" s="15">
+      <c r="C130" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/11-Web_Messaging", "Web Messaging")</f>
         <v/>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="16" t="inlineStr">
         <is>
           <t>- Assess the security of the message's origin.
 - Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F129" s="18" t="n"/>
-    </row>
-    <row r="130" ht="82.5" customHeight="1" s="82">
-      <c r="A130" s="19" t="n"/>
-      <c r="B130" s="34" t="inlineStr">
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="n"/>
+    </row>
+    <row r="131" ht="82.5" customHeight="1" s="82">
+      <c r="A131" s="19" t="n"/>
+      <c r="B131" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-12</t>
         </is>
       </c>
-      <c r="C130" s="15">
+      <c r="C131" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/12-Browser_Storage", "Browser Storage")</f>
         <v/>
       </c>
-      <c r="D130" s="16" t="inlineStr">
+      <c r="D131" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the site is storing sensitive data in client-side storage.
 - The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F130" s="18" t="n"/>
-    </row>
-    <row r="131" ht="49.5" customHeight="1" s="82">
-      <c r="A131" s="19" t="n"/>
-      <c r="B131" s="34" t="inlineStr">
+      <c r="E131" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F131" s="18" t="n"/>
+    </row>
+    <row r="132" ht="49.5" customHeight="1" s="82">
+      <c r="A132" s="19" t="n"/>
+      <c r="B132" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-13</t>
         </is>
       </c>
-      <c r="C131" s="15">
+      <c r="C132" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/13-Cross_Site_Script_Inclusion", "Cross Site Script Inclusion")</f>
         <v/>
       </c>
-      <c r="D131" s="16" t="inlineStr">
+      <c r="D132" s="16" t="inlineStr">
         <is>
           <t>- Locate sensitive data across the system.
 - Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
-      <c r="E131" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F131" s="18" t="n"/>
-    </row>
-    <row r="132" ht="16.5" customHeight="1" s="82">
-      <c r="A132" s="19" t="n"/>
-      <c r="B132" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D132" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E132" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4469,108 +4473,108 @@
       </c>
       <c r="F132" s="18" t="n"/>
     </row>
-    <row r="133" ht="99" customHeight="1" s="82">
+    <row r="133" ht="16.5" customHeight="1" s="82">
       <c r="A133" s="19" t="n"/>
       <c r="B133" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-14</t>
+        </is>
+      </c>
+      <c r="C133" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
+        <v/>
+      </c>
+      <c r="D133" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="n"/>
+    </row>
+    <row r="134" ht="99" customHeight="1" s="82">
+      <c r="A134" s="19" t="n"/>
+      <c r="B134" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-15</t>
         </is>
       </c>
-      <c r="C133" s="15">
+      <c r="C134" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/15-Client-Side_Template_Injection", "Client-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D133" s="16" t="inlineStr">
+      <c r="D134" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F133" s="18" t="n"/>
-    </row>
-    <row r="134" ht="15" customHeight="1" s="82">
-      <c r="A134" s="97" t="n"/>
-      <c r="B134" s="98" t="n"/>
-      <c r="C134" s="99" t="n"/>
-      <c r="D134" s="99" t="n"/>
-      <c r="E134" s="99" t="n"/>
-      <c r="F134" s="99" t="n"/>
-    </row>
-    <row r="135" ht="47.25" customHeight="1" s="82">
-      <c r="A135" s="9" t="n"/>
-      <c r="B135" s="100" t="inlineStr">
+      <c r="E134" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F134" s="18" t="n"/>
+    </row>
+    <row r="135" ht="15" customHeight="1" s="82">
+      <c r="A135" s="97" t="n"/>
+      <c r="B135" s="98" t="n"/>
+      <c r="C135" s="99" t="n"/>
+      <c r="D135" s="99" t="n"/>
+      <c r="E135" s="99" t="n"/>
+      <c r="F135" s="99" t="n"/>
+    </row>
+    <row r="136" ht="47.25" customHeight="1" s="82">
+      <c r="A136" s="9" t="n"/>
+      <c r="B136" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C135" s="101" t="inlineStr">
+      <c r="C136" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D135" s="101" t="inlineStr">
+      <c r="D136" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E135" s="101" t="inlineStr">
+      <c r="E136" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F135" s="101" t="inlineStr">
+      <c r="F136" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="99" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
+    <row r="137" ht="99" customHeight="1" s="82">
+      <c r="A137" s="19" t="n"/>
+      <c r="B137" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C136" s="15">
+      <c r="C137" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D136" s="16" t="inlineStr">
+      <c r="D137" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E136" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F136" s="18" t="n"/>
-    </row>
-    <row r="137" ht="66" customHeight="1" s="82">
-      <c r="A137" s="19" t="n"/>
-      <c r="B137" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-02</t>
-        </is>
-      </c>
-      <c r="C137" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D137" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
       <c r="E137" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4578,47 +4582,47 @@
       </c>
       <c r="F137" s="18" t="n"/>
     </row>
-    <row r="138" ht="132" customHeight="1" s="82">
+    <row r="138" ht="66" customHeight="1" s="82">
       <c r="A138" s="19" t="n"/>
       <c r="B138" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C138" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D138" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
+      <c r="E138" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F138" s="18" t="n"/>
+    </row>
+    <row r="139" ht="132" customHeight="1" s="82">
+      <c r="A139" s="19" t="n"/>
+      <c r="B139" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C138" s="15">
+      <c r="C139" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Excessive_Data_Exposure", "Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D138" s="16" t="inlineStr">
+      <c r="D139" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E138" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F138" s="18" t="n"/>
-    </row>
-    <row r="139" ht="82.5" customHeight="1" s="82">
-      <c r="A139" s="19" t="n"/>
-      <c r="B139" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-04</t>
-        </is>
-      </c>
-      <c r="C139" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D139" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
       <c r="E139" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4626,38 +4630,61 @@
       </c>
       <c r="F139" s="18" t="n"/>
     </row>
-    <row r="140" ht="66" customHeight="1" s="82">
+    <row r="140" ht="82.5" customHeight="1" s="82">
       <c r="A140" s="19" t="n"/>
       <c r="B140" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C140" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D140" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="66" customHeight="1" s="82">
+      <c r="A141" s="19" t="n"/>
+      <c r="B141" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C140" s="15">
+      <c r="C141" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-GraphQL", "GraphQL")</f>
         <v/>
       </c>
-      <c r="D140" s="16" t="inlineStr">
+      <c r="D141" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="82">
-      <c r="A141" s="97" t="n"/>
-      <c r="B141" s="98" t="n"/>
-      <c r="C141" s="99" t="n"/>
-      <c r="D141" s="99" t="n"/>
-      <c r="E141" s="99" t="n"/>
-      <c r="F141" s="99" t="n"/>
+      <c r="E141" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F141" s="18" t="n"/>
+    </row>
+    <row r="142" ht="15" customHeight="1" s="82">
+      <c r="A142" s="97" t="n"/>
+      <c r="B142" s="98" t="n"/>
+      <c r="C142" s="99" t="n"/>
+      <c r="D142" s="99" t="n"/>
+      <c r="E142" s="99" t="n"/>
+      <c r="F142" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4674,7 +4701,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F141">
+  <conditionalFormatting sqref="B4:F142">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4686,7 +4713,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E99 E100 E103 E104 E105 E106 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-18 (#1536)
Updates based on OWASP/wstg@8b3011c
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -2120,107 +2120,111 @@
       </c>
       <c r="F30" s="18" t="n"/>
     </row>
-    <row r="31" ht="15" customHeight="1" s="82">
-      <c r="A31" s="97" t="n"/>
-      <c r="B31" s="98" t="n"/>
-      <c r="C31" s="99" t="n"/>
-      <c r="D31" s="99" t="n"/>
-      <c r="E31" s="99" t="n"/>
-      <c r="F31" s="99" t="n"/>
-    </row>
-    <row r="32" ht="47.25" customHeight="1" s="82">
-      <c r="A32" s="9" t="n"/>
-      <c r="B32" s="100" t="inlineStr">
+    <row r="31" ht="247.5" customHeight="1" s="82">
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CONF-15</t>
+        </is>
+      </c>
+      <c r="C31" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/15-Feature_Flag_Security_Bypass", "Feature Flag Security Bypass")</f>
+        <v/>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>- Identify feature flags and kill-switches that control security-relevant functionality.
+- Determine whether feature flag states can be manipulated by an unauthorized client, and verify that backend security controls remain enforced independently of client-side flag state.
+- Verify that security controls remain consistently enforced across flag transitions, rollbacks, staged deployments, and services or instances, including whether stale security assertions or session state can be reused after a transition.
+- Evaluate fail-safe behavior when the feature flag service is unavailable.
+- Identify sensitive information exposed through feature flag configurations, and stale flags that may expose deprecated or unpatched code paths.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="82">
+      <c r="A32" s="97" t="n"/>
+      <c r="B32" s="98" t="n"/>
+      <c r="C32" s="99" t="n"/>
+      <c r="D32" s="99" t="n"/>
+      <c r="E32" s="99" t="n"/>
+      <c r="F32" s="99" t="n"/>
+    </row>
+    <row r="33" ht="47.25" customHeight="1" s="82">
+      <c r="A33" s="9" t="n"/>
+      <c r="B33" s="100" t="inlineStr">
         <is>
           <t>Identity Management</t>
         </is>
       </c>
-      <c r="C32" s="101" t="inlineStr">
+      <c r="C33" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D32" s="101" t="inlineStr">
+      <c r="D33" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E32" s="101" t="inlineStr">
+      <c r="E33" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F32" s="101" t="inlineStr">
+      <c r="F33" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="66" customHeight="1" s="82">
-      <c r="A33" s="19" t="n"/>
-      <c r="B33" s="34" t="inlineStr">
+    <row r="34" ht="66" customHeight="1" s="82">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-01</t>
         </is>
       </c>
-      <c r="C33" s="15">
+      <c r="C34" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/01-Role_Definitions", "Role Definitions")</f>
         <v/>
       </c>
-      <c r="D33" s="16" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>- Identify and document roles used by the application.
 - Attempt to switch, change, or access another role.
 - Review the granularity of the roles and the needs behind the permissions given.</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F33" s="18" t="n"/>
-    </row>
-    <row r="34" ht="49.5" customHeight="1" s="82">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="34" t="inlineStr">
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F34" s="18" t="n"/>
+    </row>
+    <row r="35" ht="49.5" customHeight="1" s="82">
+      <c r="A35" s="19" t="n"/>
+      <c r="B35" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-02</t>
         </is>
       </c>
-      <c r="C34" s="15">
+      <c r="C35" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/02-User_Registration_Process", "User Registration Process")</f>
         <v/>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>- Verify that the identity requirements for user registration are aligned with business and security requirements.
 - Validate the registration process.</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F34" s="18" t="n"/>
-    </row>
-    <row r="35" ht="33" customHeight="1" s="82">
-      <c r="A35" s="19" t="n"/>
-      <c r="B35" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-IDNT-03</t>
-        </is>
-      </c>
-      <c r="C35" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
-        <v/>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>- Verify which accounts may provision other accounts and of what type.</t>
-        </is>
-      </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2228,127 +2232,126 @@
       </c>
       <c r="F35" s="18" t="n"/>
     </row>
-    <row r="36" ht="49.5" customHeight="1" s="82">
+    <row r="36" ht="33" customHeight="1" s="82">
       <c r="A36" s="19" t="n"/>
       <c r="B36" s="34" t="inlineStr">
         <is>
+          <t>WSTG-IDNT-03</t>
+        </is>
+      </c>
+      <c r="C36" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
+        <v/>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>- Verify which accounts may provision other accounts and of what type.</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="n"/>
+    </row>
+    <row r="37" ht="49.5" customHeight="1" s="82">
+      <c r="A37" s="19" t="n"/>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
           <t>WSTG-IDNT-04</t>
         </is>
       </c>
-      <c r="C36" s="15">
+      <c r="C37" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/04-Account_Enumeration_and_Guessable_User_Account", "Account Enumeration and Guessable User Account")</f>
         <v/>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D37" s="16" t="inlineStr">
         <is>
           <t>- Review processes that pertain to user identification (*e.g.* registration, login, etc.).
 - Enumerate users where possible through response analysis.</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="n"/>
-    </row>
-    <row r="37" ht="16.5" customHeight="1" s="82">
-      <c r="A37" s="19" t="n"/>
-      <c r="B37" s="34" t="inlineStr">
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F37" s="18" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="82">
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-05</t>
         </is>
       </c>
-      <c r="C37" s="15">
+      <c r="C38" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/05-Weak_or_Unenforced_Username_Policy", "Weak or Unenforced Username Policy")</f>
         <v/>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D38" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E37" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F37" s="18" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="82">
-      <c r="A38" s="97" t="n"/>
-      <c r="B38" s="98" t="n"/>
-      <c r="C38" s="99" t="n"/>
-      <c r="D38" s="99" t="n"/>
-      <c r="E38" s="99" t="n"/>
-      <c r="F38" s="99" t="n"/>
-    </row>
-    <row r="39" ht="47.25" customHeight="1" s="82">
-      <c r="A39" s="9" t="n"/>
-      <c r="B39" s="100" t="inlineStr">
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F38" s="18" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="82">
+      <c r="A39" s="97" t="n"/>
+      <c r="B39" s="98" t="n"/>
+      <c r="C39" s="99" t="n"/>
+      <c r="D39" s="99" t="n"/>
+      <c r="E39" s="99" t="n"/>
+      <c r="F39" s="99" t="n"/>
+    </row>
+    <row r="40" ht="47.25" customHeight="1" s="82">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="100" t="inlineStr">
         <is>
           <t>Authentication</t>
         </is>
       </c>
-      <c r="C39" s="101" t="inlineStr">
+      <c r="C40" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D39" s="101" t="inlineStr">
+      <c r="D40" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E39" s="101" t="inlineStr">
+      <c r="E40" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F39" s="101" t="inlineStr">
+      <c r="F40" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="33" customHeight="1" s="82">
-      <c r="A40" s="19" t="n"/>
-      <c r="B40" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-01</t>
-        </is>
-      </c>
-      <c r="C40" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
-        <v/>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E40" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F40" s="18" t="n"/>
-    </row>
-    <row r="41" ht="66" customHeight="1" s="82">
+    <row r="41" ht="33" customHeight="1" s="82">
       <c r="A41" s="19" t="n"/>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-02</t>
+          <t>WSTG-ATHN-01</t>
         </is>
       </c>
       <c r="C41" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the application has any user accounts with default passwords.
-- Review whether new user accounts are created with weak or predictable passwords.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">
@@ -2362,40 +2365,41 @@
       <c r="A42" s="19" t="n"/>
       <c r="B42" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-02</t>
+        </is>
+      </c>
+      <c r="C42" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
+        <v/>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether the application has any user accounts with default passwords.
+- Review whether new user accounts are created with weak or predictable passwords.</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F42" s="18" t="n"/>
+    </row>
+    <row r="43" ht="66" customHeight="1" s="82">
+      <c r="A43" s="19" t="n"/>
+      <c r="B43" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-03</t>
         </is>
       </c>
-      <c r="C42" s="15">
+      <c r="C43" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/03-Weak_Lock_Out_Mechanism", "Weak Lock Out Mechanism")</f>
         <v/>
       </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="D43" s="16" t="inlineStr">
         <is>
           <t>- Evaluate the account lockout mechanism's ability to mitigate brute force password guessing.
 - Evaluate the unlock mechanism's resistance to unauthorized account unlocking.</t>
-        </is>
-      </c>
-      <c r="E42" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F42" s="18" t="n"/>
-    </row>
-    <row r="43" ht="33" customHeight="1" s="82">
-      <c r="A43" s="19" t="n"/>
-      <c r="B43" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-04</t>
-        </is>
-      </c>
-      <c r="C43" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
-        <v/>
-      </c>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>- Ensure that authentication is applied across all services that require it.</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
@@ -2409,16 +2413,16 @@
       <c r="A44" s="19" t="n"/>
       <c r="B44" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-05</t>
+          <t>WSTG-ATHN-04</t>
         </is>
       </c>
       <c r="C44" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
+          <t>- Ensure that authentication is applied across all services that require it.</t>
         </is>
       </c>
       <c r="E44" s="18" t="inlineStr">
@@ -2428,46 +2432,46 @@
       </c>
       <c r="F44" s="18" t="n"/>
     </row>
-    <row r="45" ht="49.5" customHeight="1" s="82">
+    <row r="45" ht="33" customHeight="1" s="82">
       <c r="A45" s="19" t="n"/>
       <c r="B45" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-05</t>
+        </is>
+      </c>
+      <c r="C45" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
+        <v/>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F45" s="18" t="n"/>
+    </row>
+    <row r="46" ht="49.5" customHeight="1" s="82">
+      <c r="A46" s="19" t="n"/>
+      <c r="B46" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-06</t>
         </is>
       </c>
-      <c r="C45" s="15">
+      <c r="C46" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/06-Browser_Cache_Weaknesses", "Browser Cache Weaknesses")</f>
         <v/>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>- Review if the application stores sensitive information on the client-side.
 - Review if access can occur without authorization.</t>
         </is>
       </c>
-      <c r="E45" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F45" s="18" t="n"/>
-    </row>
-    <row r="46" ht="66" customHeight="1" s="82">
-      <c r="A46" s="19" t="n"/>
-      <c r="B46" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-07</t>
-        </is>
-      </c>
-      <c r="C46" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
-        <v/>
-      </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
-        </is>
-      </c>
       <c r="E46" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2475,46 +2479,46 @@
       </c>
       <c r="F46" s="18" t="n"/>
     </row>
-    <row r="47" ht="49.5" customHeight="1" s="82">
+    <row r="47" ht="66" customHeight="1" s="82">
       <c r="A47" s="19" t="n"/>
       <c r="B47" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-07</t>
+        </is>
+      </c>
+      <c r="C47" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
+        <v/>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
+        </is>
+      </c>
+      <c r="E47" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F47" s="18" t="n"/>
+    </row>
+    <row r="48" ht="49.5" customHeight="1" s="82">
+      <c r="A48" s="19" t="n"/>
+      <c r="B48" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-08</t>
         </is>
       </c>
-      <c r="C47" s="15">
+      <c r="C48" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/08-Weak_Security_Question_Answer", "Weak Security Question Answer")</f>
         <v/>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D48" s="16" t="inlineStr">
         <is>
           <t>- Determine the complexity and how straight-forward the questions are.
 - Assess possible user answers and brute force capabilities.</t>
         </is>
       </c>
-      <c r="E47" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F47" s="18" t="n"/>
-    </row>
-    <row r="48" ht="33" customHeight="1" s="82">
-      <c r="A48" s="19" t="n"/>
-      <c r="B48" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-09</t>
-        </is>
-      </c>
-      <c r="C48" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
-        <v/>
-      </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
-        </is>
-      </c>
       <c r="E48" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2522,131 +2526,131 @@
       </c>
       <c r="F48" s="18" t="n"/>
     </row>
-    <row r="49" ht="49.5" customHeight="1" s="82">
+    <row r="49" ht="33" customHeight="1" s="82">
       <c r="A49" s="19" t="n"/>
       <c r="B49" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHN-09</t>
+        </is>
+      </c>
+      <c r="C49" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
+        <v/>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F49" s="18" t="n"/>
+    </row>
+    <row r="50" ht="49.5" customHeight="1" s="82">
+      <c r="A50" s="19" t="n"/>
+      <c r="B50" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHN-10</t>
         </is>
       </c>
-      <c r="C49" s="15">
+      <c r="C50" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/10-Weaker_Authentication_in_Alternative_Channel", "Weaker Authentication in Alternative Channel")</f>
         <v/>
       </c>
-      <c r="D49" s="16" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>- Identify alternative authentication channels.
 - Assess the security measures used and if any bypasses exists on the alternative channels.</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F49" s="18" t="n"/>
-    </row>
-    <row r="50" ht="66" customHeight="1" s="82">
-      <c r="A50" s="19" t="n"/>
-      <c r="B50" s="34" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="n"/>
+    </row>
+    <row r="51" ht="66" customHeight="1" s="82">
+      <c r="A51" s="19" t="n"/>
+      <c r="B51" s="34" t="inlineStr">
         <is>
           <t>WSTG-ATHN-11</t>
         </is>
       </c>
-      <c r="C50" s="15">
+      <c r="C51" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/11-Multi-Factor_Authentication", "Multi-Factor Authentication (MFA)")</f>
         <v/>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>- Identify the type of MFA used by the application.
 - Determine whether the MFA implementation is robust and secure.
 - Attempt to bypass the MFA.</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="82">
-      <c r="A51" s="97" t="n"/>
-      <c r="B51" s="98" t="n"/>
-      <c r="C51" s="99" t="n"/>
-      <c r="D51" s="99" t="n"/>
-      <c r="E51" s="99" t="n"/>
-      <c r="F51" s="99" t="n"/>
-    </row>
-    <row r="52" ht="47.25" customHeight="1" s="82">
-      <c r="A52" s="9" t="n"/>
-      <c r="B52" s="100" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F51" s="18" t="n"/>
+    </row>
+    <row r="52" ht="15" customHeight="1" s="82">
+      <c r="A52" s="97" t="n"/>
+      <c r="B52" s="98" t="n"/>
+      <c r="C52" s="99" t="n"/>
+      <c r="D52" s="99" t="n"/>
+      <c r="E52" s="99" t="n"/>
+      <c r="F52" s="99" t="n"/>
+    </row>
+    <row r="53" ht="47.25" customHeight="1" s="82">
+      <c r="A53" s="9" t="n"/>
+      <c r="B53" s="100" t="inlineStr">
         <is>
           <t>Authorization</t>
         </is>
       </c>
-      <c r="C52" s="101" t="inlineStr">
+      <c r="C53" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D52" s="101" t="inlineStr">
+      <c r="D53" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E52" s="101" t="inlineStr">
+      <c r="E53" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F52" s="101" t="inlineStr">
+      <c r="F53" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="49.5" customHeight="1" s="82">
-      <c r="A53" s="19" t="n"/>
-      <c r="B53" s="34" t="inlineStr">
+    <row r="54" ht="49.5" customHeight="1" s="82">
+      <c r="A54" s="19" t="n"/>
+      <c r="B54" s="34" t="inlineStr">
         <is>
           <t>WSTG-ATHZ-01</t>
         </is>
       </c>
-      <c r="C53" s="15">
+      <c r="C54" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/01-Directory_Traversal_File_Include", "Directory Traversal File Include")</f>
         <v/>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D54" s="16" t="inlineStr">
         <is>
           <t>- Identify injection points that pertain to path traversal.
 - Assess bypassing techniques and identify the extent of path traversal.</t>
         </is>
       </c>
-      <c r="E53" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F53" s="18" t="n"/>
-    </row>
-    <row r="54" ht="33" customHeight="1" s="82">
-      <c r="A54" s="19" t="n"/>
-      <c r="B54" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHZ-02</t>
-        </is>
-      </c>
-      <c r="C54" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
-        <v/>
-      </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
-        </is>
-      </c>
       <c r="E54" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2654,21 +2658,20 @@
       </c>
       <c r="F54" s="18" t="n"/>
     </row>
-    <row r="55" ht="49.5" customHeight="1" s="82">
+    <row r="55" ht="33" customHeight="1" s="82">
       <c r="A55" s="19" t="n"/>
       <c r="B55" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-03</t>
+          <t>WSTG-ATHZ-02</t>
         </is>
       </c>
       <c r="C55" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points related to privilege manipulation.
-- Fuzz or otherwise attempt to bypass security measures.</t>
+          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
         </is>
       </c>
       <c r="E55" s="18" t="inlineStr">
@@ -2682,126 +2685,127 @@
       <c r="A56" s="19" t="n"/>
       <c r="B56" s="34" t="inlineStr">
         <is>
+          <t>WSTG-ATHZ-03</t>
+        </is>
+      </c>
+      <c r="C56" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
+        <v/>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>- Identify injection points related to privilege manipulation.
+- Fuzz or otherwise attempt to bypass security measures.</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="n"/>
+    </row>
+    <row r="57" ht="49.5" customHeight="1" s="82">
+      <c r="A57" s="19" t="n"/>
+      <c r="B57" s="34" t="inlineStr">
+        <is>
           <t>WSTG-ATHZ-04</t>
         </is>
       </c>
-      <c r="C56" s="15">
+      <c r="C57" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/04-Insecure_Direct_Object_References", "Insecure Direct Object References")</f>
         <v/>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>- Identify points where object references may occur.
 - Assess the access control measures and if they're vulnerable to IDOR.</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="n"/>
-    </row>
-    <row r="57" ht="33" customHeight="1" s="82">
-      <c r="A57" s="19" t="n"/>
-      <c r="B57" s="34" t="inlineStr">
+      <c r="E57" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="n"/>
+    </row>
+    <row r="58" ht="33" customHeight="1" s="82">
+      <c r="A58" s="19" t="n"/>
+      <c r="B58" s="34" t="inlineStr">
         <is>
           <t>WSTG-ATHZ-05</t>
         </is>
       </c>
-      <c r="C57" s="15">
+      <c r="C58" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/05-OAuth_Weaknesses", "OAuth Weaknesses")</f>
         <v/>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>- Determine if OAuth2 implementation is vulnerable or using a deprecated or custom implementation.</t>
         </is>
       </c>
-      <c r="E57" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F57" s="18" t="n"/>
-    </row>
-    <row r="58" ht="15" customHeight="1" s="82">
-      <c r="A58" s="97" t="n"/>
-      <c r="B58" s="98" t="n"/>
-      <c r="C58" s="99" t="n"/>
-      <c r="D58" s="99" t="n"/>
-      <c r="E58" s="99" t="n"/>
-      <c r="F58" s="99" t="n"/>
-    </row>
-    <row r="59" ht="47.25" customHeight="1" s="82">
-      <c r="A59" s="9" t="n"/>
-      <c r="B59" s="100" t="inlineStr">
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="n"/>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="82">
+      <c r="A59" s="97" t="n"/>
+      <c r="B59" s="98" t="n"/>
+      <c r="C59" s="99" t="n"/>
+      <c r="D59" s="99" t="n"/>
+      <c r="E59" s="99" t="n"/>
+      <c r="F59" s="99" t="n"/>
+    </row>
+    <row r="60" ht="47.25" customHeight="1" s="82">
+      <c r="A60" s="9" t="n"/>
+      <c r="B60" s="100" t="inlineStr">
         <is>
           <t>Session Management</t>
         </is>
       </c>
-      <c r="C59" s="101" t="inlineStr">
+      <c r="C60" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D59" s="101" t="inlineStr">
+      <c r="D60" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E59" s="101" t="inlineStr">
+      <c r="E60" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F59" s="101" t="inlineStr">
+      <c r="F60" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="99" customHeight="1" s="82">
-      <c r="A60" s="19" t="n"/>
-      <c r="B60" s="34" t="inlineStr">
+    <row r="61" ht="99" customHeight="1" s="82">
+      <c r="A61" s="19" t="n"/>
+      <c r="B61" s="34" t="inlineStr">
         <is>
           <t>WSTG-SESS-01</t>
         </is>
       </c>
-      <c r="C60" s="15">
+      <c r="C61" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/01-Session_Management_Schema", "Session Management Schema")</f>
         <v/>
       </c>
-      <c r="D60" s="16" t="inlineStr">
+      <c r="D61" s="16" t="inlineStr">
         <is>
           <t>- Gather session tokens, for the same user and for different users where possible.
 - Analyze and ensure that enough randomness exists to stop session forging attacks.
 - Modify cookies that are not signed and contain information that can be manipulated.</t>
         </is>
       </c>
-      <c r="E60" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F60" s="18" t="n"/>
-    </row>
-    <row r="61" ht="33" customHeight="1" s="82">
-      <c r="A61" s="19" t="n"/>
-      <c r="B61" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-02</t>
-        </is>
-      </c>
-      <c r="C61" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
-        <v/>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>- Ensure that the proper security configuration is set for cookies.</t>
-        </is>
-      </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2813,67 +2817,67 @@
       <c r="A62" s="19" t="n"/>
       <c r="B62" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-02</t>
+        </is>
+      </c>
+      <c r="C62" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
+        <v/>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>- Ensure that the proper security configuration is set for cookies.</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="n"/>
+    </row>
+    <row r="63" ht="33" customHeight="1" s="82">
+      <c r="A63" s="19" t="n"/>
+      <c r="B63" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-03</t>
         </is>
       </c>
-      <c r="C62" s="15">
+      <c r="C63" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/03-Session_Fixation", "Session Fixation")</f>
         <v/>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D63" s="16" t="inlineStr">
         <is>
           <t>- Analyze the authentication mechanism and its flow.
 - Force cookies and assess the impact.</t>
         </is>
       </c>
-      <c r="E62" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F62" s="18" t="n"/>
-    </row>
-    <row r="63" ht="49.5" customHeight="1" s="82">
-      <c r="A63" s="19" t="n"/>
-      <c r="B63" s="34" t="inlineStr">
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="n"/>
+    </row>
+    <row r="64" ht="49.5" customHeight="1" s="82">
+      <c r="A64" s="19" t="n"/>
+      <c r="B64" s="34" t="inlineStr">
         <is>
           <t>WSTG-SESS-04</t>
         </is>
       </c>
-      <c r="C63" s="15">
+      <c r="C64" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/04-Exposed_Session_Variables", "Exposed Session Variables")</f>
         <v/>
       </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>- Ensure that proper encryption is implemented.
 - Review the caching configuration.
 - Assess the channel and methods' security.</t>
         </is>
       </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F63" s="18" t="n"/>
-    </row>
-    <row r="64" ht="33" customHeight="1" s="82">
-      <c r="A64" s="19" t="n"/>
-      <c r="B64" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-05</t>
-        </is>
-      </c>
-      <c r="C64" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
-        <v/>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
-        </is>
-      </c>
       <c r="E64" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2881,46 +2885,46 @@
       </c>
       <c r="F64" s="18" t="n"/>
     </row>
-    <row r="65" ht="49.5" customHeight="1" s="82">
+    <row r="65" ht="33" customHeight="1" s="82">
       <c r="A65" s="19" t="n"/>
       <c r="B65" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-05</t>
+        </is>
+      </c>
+      <c r="C65" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
+        <v/>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="n"/>
+    </row>
+    <row r="66" ht="49.5" customHeight="1" s="82">
+      <c r="A66" s="19" t="n"/>
+      <c r="B66" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-06</t>
         </is>
       </c>
-      <c r="C65" s="15">
+      <c r="C66" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/06-Logout_Functionality", "Logout Functionality")</f>
         <v/>
       </c>
-      <c r="D65" s="16" t="inlineStr">
+      <c r="D66" s="16" t="inlineStr">
         <is>
           <t>- Assess the logout UI.
 - Analyze the session timeout and if the session is properly killed after logout.</t>
         </is>
       </c>
-      <c r="E65" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F65" s="18" t="n"/>
-    </row>
-    <row r="66" ht="16.5" customHeight="1" s="82">
-      <c r="A66" s="19" t="n"/>
-      <c r="B66" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-07</t>
-        </is>
-      </c>
-      <c r="C66" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
-        <v/>
-      </c>
-      <c r="D66" s="16" t="inlineStr">
-        <is>
-          <t>- Validate that a hard session timeout exists.</t>
-        </is>
-      </c>
       <c r="E66" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2928,21 +2932,20 @@
       </c>
       <c r="F66" s="18" t="n"/>
     </row>
-    <row r="67" ht="33" customHeight="1" s="82">
+    <row r="67" ht="16.5" customHeight="1" s="82">
       <c r="A67" s="19" t="n"/>
       <c r="B67" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-08</t>
+          <t>WSTG-SESS-07</t>
         </is>
       </c>
       <c r="C67" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
         <v/>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>- Identify all session variables.
-- Break the logical flow of session generation.</t>
+          <t>- Validate that a hard session timeout exists.</t>
         </is>
       </c>
       <c r="E67" s="18" t="inlineStr">
@@ -2956,41 +2959,41 @@
       <c r="A68" s="19" t="n"/>
       <c r="B68" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-08</t>
+        </is>
+      </c>
+      <c r="C68" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
+        <v/>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>- Identify all session variables.
+- Break the logical flow of session generation.</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="n"/>
+    </row>
+    <row r="69" ht="33" customHeight="1" s="82">
+      <c r="A69" s="19" t="n"/>
+      <c r="B69" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-09</t>
         </is>
       </c>
-      <c r="C68" s="15">
+      <c r="C69" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/09-Session_Hijacking", "Session Hijacking")</f>
         <v/>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D69" s="16" t="inlineStr">
         <is>
           <t>- Identify vulnerable session cookies.
 - Hijack vulnerable cookies and assess the risk level.</t>
-        </is>
-      </c>
-      <c r="E68" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F68" s="18" t="n"/>
-    </row>
-    <row r="69" ht="49.5" customHeight="1" s="82">
-      <c r="A69" s="19" t="n"/>
-      <c r="B69" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-10</t>
-        </is>
-      </c>
-      <c r="C69" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
-        <v/>
-      </c>
-      <c r="D69" s="16" t="inlineStr">
-        <is>
-          <t>- Determine whether the JWTs expose sensitive information.
-- Determine whether the JWTs can be tampered with or modified.</t>
         </is>
       </c>
       <c r="E69" s="18" t="inlineStr">
@@ -3004,125 +3007,126 @@
       <c r="A70" s="19" t="n"/>
       <c r="B70" s="34" t="inlineStr">
         <is>
+          <t>WSTG-SESS-10</t>
+        </is>
+      </c>
+      <c r="C70" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
+        <v/>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether the JWTs expose sensitive information.
+- Determine whether the JWTs can be tampered with or modified.</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="n"/>
+    </row>
+    <row r="71" ht="49.5" customHeight="1" s="82">
+      <c r="A71" s="19" t="n"/>
+      <c r="B71" s="34" t="inlineStr">
+        <is>
           <t>WSTG-SESS-11</t>
         </is>
       </c>
-      <c r="C70" s="15">
+      <c r="C71" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/11-Concurrent_Sessions", "Concurrent Sessions")</f>
         <v/>
       </c>
-      <c r="D70" s="16" t="inlineStr">
+      <c r="D71" s="16" t="inlineStr">
         <is>
           <t>- Evaluate the application's session management by assessing the handling of multiple active sessions for a single user account.</t>
         </is>
       </c>
-      <c r="E70" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F70" s="18" t="n"/>
-    </row>
-    <row r="71" ht="15" customHeight="1" s="82">
-      <c r="A71" s="97" t="n"/>
-      <c r="B71" s="98" t="n"/>
-      <c r="C71" s="99" t="n"/>
-      <c r="D71" s="99" t="n"/>
-      <c r="E71" s="99" t="n"/>
-      <c r="F71" s="99" t="n"/>
-    </row>
-    <row r="72" ht="47.25" customHeight="1" s="82">
-      <c r="A72" s="9" t="n"/>
-      <c r="B72" s="100" t="inlineStr">
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="n"/>
+    </row>
+    <row r="72" ht="15" customHeight="1" s="82">
+      <c r="A72" s="97" t="n"/>
+      <c r="B72" s="98" t="n"/>
+      <c r="C72" s="99" t="n"/>
+      <c r="D72" s="99" t="n"/>
+      <c r="E72" s="99" t="n"/>
+      <c r="F72" s="99" t="n"/>
+    </row>
+    <row r="73" ht="47.25" customHeight="1" s="82">
+      <c r="A73" s="9" t="n"/>
+      <c r="B73" s="100" t="inlineStr">
         <is>
           <t>Injection</t>
         </is>
       </c>
-      <c r="C72" s="101" t="inlineStr">
+      <c r="C73" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D72" s="101" t="inlineStr">
+      <c r="D73" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E72" s="101" t="inlineStr">
+      <c r="E73" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F72" s="101" t="inlineStr">
+      <c r="F73" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="49.5" customHeight="1" s="82">
-      <c r="A73" s="19" t="n"/>
-      <c r="B73" s="34" t="inlineStr">
+    <row r="74" ht="49.5" customHeight="1" s="82">
+      <c r="A74" s="19" t="n"/>
+      <c r="B74" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-01</t>
         </is>
       </c>
-      <c r="C73" s="15">
+      <c r="C74" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/01-Reflected_Cross_Site_Scripting", "Reflected Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D73" s="16" t="inlineStr">
+      <c r="D74" s="16" t="inlineStr">
         <is>
           <t>- Identify variables that are reflected in responses.
 - Assess the input they accept and the encoding that gets applied on return (if any).</t>
         </is>
       </c>
-      <c r="E73" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F73" s="18" t="n"/>
-    </row>
-    <row r="74" ht="66" customHeight="1" s="82">
-      <c r="A74" s="19" t="n"/>
-      <c r="B74" s="34" t="inlineStr">
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="n"/>
+    </row>
+    <row r="75" ht="66" customHeight="1" s="82">
+      <c r="A75" s="19" t="n"/>
+      <c r="B75" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-02</t>
         </is>
       </c>
-      <c r="C74" s="15">
+      <c r="C75" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/02-Stored_Cross_Site_Scripting", "Stored Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D74" s="16" t="inlineStr">
+      <c r="D75" s="16" t="inlineStr">
         <is>
           <t>- Identify stored input that is reflected on the client-side.
 - Assess the input they accept and the encoding that gets applied on return (if any).</t>
         </is>
       </c>
-      <c r="E74" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F74" s="18" t="n"/>
-    </row>
-    <row r="75" ht="16.5" customHeight="1" s="82">
-      <c r="A75" s="19" t="n"/>
-      <c r="B75" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-03</t>
-        </is>
-      </c>
-      <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
-        <v/>
-      </c>
-      <c r="D75" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E75" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3130,21 +3134,20 @@
       </c>
       <c r="F75" s="18" t="n"/>
     </row>
-    <row r="76" ht="49.5" customHeight="1" s="82">
+    <row r="76" ht="16.5" customHeight="1" s="82">
       <c r="A76" s="19" t="n"/>
       <c r="B76" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INJT-04</t>
+          <t>WSTG-INJT-03</t>
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>- Identify the back end and the parsing method used.
-- Assess injection points and try bypassing input filters using HPP.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E76" s="18" t="inlineStr">
@@ -3158,114 +3161,115 @@
       <c r="A77" s="19" t="n"/>
       <c r="B77" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-04</t>
+        </is>
+      </c>
+      <c r="C77" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
+        <v/>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the back end and the parsing method used.
+- Assess injection points and try bypassing input filters using HPP.</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="n"/>
+    </row>
+    <row r="78" ht="49.5" customHeight="1" s="82">
+      <c r="A78" s="19" t="n"/>
+      <c r="B78" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-05</t>
         </is>
       </c>
-      <c r="C77" s="15">
+      <c r="C78" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/05-SQL_Injection", "SQL Injection")</f>
         <v/>
       </c>
-      <c r="D77" s="16" t="inlineStr">
+      <c r="D78" s="16" t="inlineStr">
         <is>
           <t>- Identify SQL injection points.
 - Assess the severity of the injection and the level of access that can be achieved through it.</t>
         </is>
       </c>
-      <c r="E77" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F77" s="18" t="n"/>
-    </row>
-    <row r="78" ht="33" customHeight="1" s="82">
-      <c r="A78" s="19" t="n"/>
-      <c r="B78" s="34" t="inlineStr">
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="n"/>
+    </row>
+    <row r="79" ht="33" customHeight="1" s="82">
+      <c r="A79" s="19" t="n"/>
+      <c r="B79" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-06</t>
         </is>
       </c>
-      <c r="C78" s="15">
+      <c r="C79" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/06-LDAP_Injection", "LDAP Injection")</f>
         <v/>
       </c>
-      <c r="D78" s="16" t="inlineStr">
+      <c r="D79" s="16" t="inlineStr">
         <is>
           <t>- Identify LDAP injection points.
 - Assess the severity of the injection.</t>
         </is>
       </c>
-      <c r="E78" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F78" s="18" t="n"/>
-    </row>
-    <row r="79" ht="49.5" customHeight="1" s="82">
-      <c r="A79" s="19" t="n"/>
-      <c r="B79" s="34" t="inlineStr">
+      <c r="E79" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="n"/>
+    </row>
+    <row r="80" ht="49.5" customHeight="1" s="82">
+      <c r="A80" s="19" t="n"/>
+      <c r="B80" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-07</t>
         </is>
       </c>
-      <c r="C79" s="15">
+      <c r="C80" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/07-XML_Injection", "XML Injection")</f>
         <v/>
       </c>
-      <c r="D79" s="16" t="inlineStr">
+      <c r="D80" s="16" t="inlineStr">
         <is>
           <t>- Identify XML injection points.
 - Assess the types of exploits that can be attained and their severities.</t>
         </is>
       </c>
-      <c r="E79" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F79" s="18" t="n"/>
-    </row>
-    <row r="80" ht="33" customHeight="1" s="82">
-      <c r="A80" s="19" t="n"/>
-      <c r="B80" s="34" t="inlineStr">
+      <c r="E80" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="n"/>
+    </row>
+    <row r="81" ht="33" customHeight="1" s="82">
+      <c r="A81" s="19" t="n"/>
+      <c r="B81" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-08</t>
         </is>
       </c>
-      <c r="C80" s="15">
+      <c r="C81" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/08-SSI_Injection", "SSI Injection")</f>
         <v/>
       </c>
-      <c r="D80" s="16" t="inlineStr">
+      <c r="D81" s="16" t="inlineStr">
         <is>
           <t>- Identify SSI injection points.
 - Assess the severity of the injection.</t>
         </is>
       </c>
-      <c r="E80" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F80" s="18" t="n"/>
-    </row>
-    <row r="81" ht="16.5" customHeight="1" s="82">
-      <c r="A81" s="19" t="n"/>
-      <c r="B81" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-09</t>
-        </is>
-      </c>
-      <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
-        <v/>
-      </c>
-      <c r="D81" s="16" t="inlineStr">
-        <is>
-          <t>- Identify XPATH injection points.</t>
-        </is>
-      </c>
       <c r="E81" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3273,95 +3277,95 @@
       </c>
       <c r="F81" s="18" t="n"/>
     </row>
-    <row r="82" ht="66" customHeight="1" s="82">
+    <row r="82" ht="16.5" customHeight="1" s="82">
       <c r="A82" s="19" t="n"/>
       <c r="B82" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-09</t>
+        </is>
+      </c>
+      <c r="C82" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
+        <v/>
+      </c>
+      <c r="D82" s="16" t="inlineStr">
+        <is>
+          <t>- Identify XPATH injection points.</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="n"/>
+    </row>
+    <row r="83" ht="66" customHeight="1" s="82">
+      <c r="A83" s="19" t="n"/>
+      <c r="B83" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-10</t>
         </is>
       </c>
-      <c r="C82" s="15">
+      <c r="C83" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/10-IMAP_SMTP_Injection", "IMAP SMTP Injection")</f>
         <v/>
       </c>
-      <c r="D82" s="16" t="inlineStr">
+      <c r="D83" s="16" t="inlineStr">
         <is>
           <t>- Identify IMAP/SMTP injection points.
 - Understand the data flow and deployment structure of the system.
 - Assess the injection impacts.</t>
         </is>
       </c>
-      <c r="E82" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F82" s="18" t="n"/>
-    </row>
-    <row r="83" ht="49.5" customHeight="1" s="82">
-      <c r="A83" s="19" t="n"/>
-      <c r="B83" s="34" t="inlineStr">
+      <c r="E83" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F83" s="18" t="n"/>
+    </row>
+    <row r="84" ht="49.5" customHeight="1" s="82">
+      <c r="A84" s="19" t="n"/>
+      <c r="B84" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-11</t>
         </is>
       </c>
-      <c r="C83" s="15">
+      <c r="C84" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/11-Code_Injection", "Code Injection")</f>
         <v/>
       </c>
-      <c r="D83" s="16" t="inlineStr">
+      <c r="D84" s="16" t="inlineStr">
         <is>
           <t>- Identify injection points where you can inject code into the application.
 - Assess the injection severity.</t>
         </is>
       </c>
-      <c r="E83" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F83" s="18" t="n"/>
-    </row>
-    <row r="84" ht="33" customHeight="1" s="82">
-      <c r="A84" s="19" t="n"/>
-      <c r="B84" s="34" t="inlineStr">
+      <c r="E84" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F84" s="18" t="n"/>
+    </row>
+    <row r="85" ht="33" customHeight="1" s="82">
+      <c r="A85" s="19" t="n"/>
+      <c r="B85" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-12</t>
         </is>
       </c>
-      <c r="C84" s="15">
+      <c r="C85" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/12-Command_Injection", "Command Injection")</f>
         <v/>
       </c>
-      <c r="D84" s="16" t="inlineStr">
+      <c r="D85" s="16" t="inlineStr">
         <is>
           <t>- Identify and assess command injection points.
 - Bypass special characters and OS commands filter.</t>
         </is>
       </c>
-      <c r="E84" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F84" s="18" t="n"/>
-    </row>
-    <row r="85" ht="49.5" customHeight="1" s="82">
-      <c r="A85" s="19" t="n"/>
-      <c r="B85" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-13</t>
-        </is>
-      </c>
-      <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
-        <v/>
-      </c>
-      <c r="D85" s="16" t="inlineStr">
-        <is>
-          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
-        </is>
-      </c>
       <c r="E85" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3369,68 +3373,91 @@
       </c>
       <c r="F85" s="18" t="n"/>
     </row>
-    <row r="86" ht="66" customHeight="1" s="82">
+    <row r="86" ht="49.5" customHeight="1" s="82">
       <c r="A86" s="19" t="n"/>
       <c r="B86" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-13</t>
+        </is>
+      </c>
+      <c r="C86" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
+        <v/>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="n"/>
+    </row>
+    <row r="87" ht="66" customHeight="1" s="82">
+      <c r="A87" s="19" t="n"/>
+      <c r="B87" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-14</t>
         </is>
       </c>
-      <c r="C86" s="15">
+      <c r="C87" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/14-Incubated_Vulnerability", "Incubated Vulnerability")</f>
         <v/>
       </c>
-      <c r="D86" s="16" t="inlineStr">
+      <c r="D87" s="16" t="inlineStr">
         <is>
           <t>- Identify injections that are stored and require a recall step to the stored injection.
 - Understand how a recall step could occur.
 - Set listeners or activate the recall step if possible.</t>
         </is>
       </c>
-      <c r="E86" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F86" s="18" t="n"/>
-    </row>
-    <row r="87" ht="115.5" customHeight="1" s="82">
-      <c r="A87" s="19" t="n"/>
-      <c r="B87" s="34" t="inlineStr">
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="n"/>
+    </row>
+    <row r="88" ht="115.5" customHeight="1" s="82">
+      <c r="A88" s="19" t="n"/>
+      <c r="B88" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-15</t>
         </is>
       </c>
-      <c r="C87" s="15">
+      <c r="C88" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/15-HTTP_Response_Splitting", "HTTP Response Splitting")</f>
         <v/>
       </c>
-      <c r="D87" s="16" t="inlineStr">
+      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>- Identify user-controlled input that is reflected into HTTP response headers.
 - Assess whether CR (`\r`) and LF (`\n`) characters can be injected into response headers.
 - Determine the potential impact of successful HTTP Response Splitting attacks, such as cache poisoning or client-side exploitation.</t>
         </is>
       </c>
-      <c r="E87" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F87" s="18" t="n"/>
-    </row>
-    <row r="88" ht="99" customHeight="1" s="82">
-      <c r="A88" s="19" t="n"/>
-      <c r="B88" s="34" t="inlineStr">
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="n"/>
+    </row>
+    <row r="89" ht="99" customHeight="1" s="82">
+      <c r="A89" s="19" t="n"/>
+      <c r="B89" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-16</t>
         </is>
       </c>
-      <c r="C88" s="15">
+      <c r="C89" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/16-HTTP_Request_Smuggling", "HTTP Request Smuggling")</f>
         <v/>
       </c>
-      <c r="D88" s="16" t="inlineStr">
+      <c r="D89" s="16" t="inlineStr">
         <is>
           <t>- Identify request boundary inconsistencies between frontend and backend components
 - Detect classic CL/TE desynchronization vulnerabilities
@@ -3439,30 +3466,6 @@
 - Confirm backend request queue poisoning</t>
         </is>
       </c>
-      <c r="E88" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F88" s="18" t="n"/>
-    </row>
-    <row r="89" ht="49.5" customHeight="1" s="82">
-      <c r="A89" s="19" t="n"/>
-      <c r="B89" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INJT-17</t>
-        </is>
-      </c>
-      <c r="C89" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
-        <v/>
-      </c>
-      <c r="D89" s="16" t="inlineStr">
-        <is>
-          <t>- Assess if the Host header is being parsed dynamically in the application.
-- Bypass security controls that rely on the header.</t>
-        </is>
-      </c>
       <c r="E89" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3474,88 +3477,112 @@
       <c r="A90" s="19" t="n"/>
       <c r="B90" s="34" t="inlineStr">
         <is>
+          <t>WSTG-INJT-17</t>
+        </is>
+      </c>
+      <c r="C90" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
+        <v/>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>- Assess if the Host header is being parsed dynamically in the application.
+- Bypass security controls that rely on the header.</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F90" s="18" t="n"/>
+    </row>
+    <row r="91" ht="49.5" customHeight="1" s="82">
+      <c r="A91" s="19" t="n"/>
+      <c r="B91" s="34" t="inlineStr">
+        <is>
           <t>WSTG-INJT-18</t>
         </is>
       </c>
-      <c r="C90" s="15">
+      <c r="C91" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/18-Server-side_Template_Injection", "Server-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="D91" s="16" t="inlineStr">
         <is>
           <t>- Detect template injection vulnerability points.
 - Identify the templating engine.
 - Build the exploit.</t>
         </is>
       </c>
-      <c r="E90" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F90" s="18" t="n"/>
-    </row>
-    <row r="91" ht="49.5" customHeight="1" s="82">
-      <c r="A91" s="19" t="n"/>
-      <c r="B91" s="34" t="inlineStr">
+      <c r="E91" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F91" s="18" t="n"/>
+    </row>
+    <row r="92" ht="49.5" customHeight="1" s="82">
+      <c r="A92" s="19" t="n"/>
+      <c r="B92" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-19</t>
         </is>
       </c>
-      <c r="C91" s="15">
+      <c r="C92" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/19-Server-Side_Request_Forgery", "Server-Side Request Forgery")</f>
         <v/>
       </c>
-      <c r="D91" s="16" t="inlineStr">
+      <c r="D92" s="16" t="inlineStr">
         <is>
           <t>- Identify SSRF injection points.
 - Test if the injection points are exploitable.
 - Asses the severity of the vulnerability.</t>
         </is>
       </c>
-      <c r="E91" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F91" s="18" t="n"/>
-    </row>
-    <row r="92" ht="49.5" customHeight="1" s="82">
-      <c r="A92" s="19" t="n"/>
-      <c r="B92" s="34" t="inlineStr">
+      <c r="E92" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F92" s="18" t="n"/>
+    </row>
+    <row r="93" ht="49.5" customHeight="1" s="82">
+      <c r="A93" s="19" t="n"/>
+      <c r="B93" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-20</t>
         </is>
       </c>
-      <c r="C92" s="15">
+      <c r="C93" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/20-Mass_Assignment", "Mass Assignment")</f>
         <v/>
       </c>
-      <c r="D92" s="16" t="inlineStr">
+      <c r="D93" s="16" t="inlineStr">
         <is>
           <t>- Identify requests that modify objects
 - Assess if it is possible to modify fields never intended to be modified from outside</t>
         </is>
       </c>
-      <c r="E92" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F92" s="18" t="n"/>
-    </row>
-    <row r="93" ht="181.5" customHeight="1" s="82">
-      <c r="A93" s="19" t="n"/>
-      <c r="B93" s="34" t="inlineStr">
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="n"/>
+    </row>
+    <row r="94" ht="181.5" customHeight="1" s="82">
+      <c r="A94" s="19" t="n"/>
+      <c r="B94" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-21</t>
         </is>
       </c>
-      <c r="C93" s="15">
+      <c r="C94" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/21-CSV_Injection", "CSV Injection")</f>
         <v/>
       </c>
-      <c r="D93" s="16" t="inlineStr">
+      <c r="D94" s="16" t="inlineStr">
         <is>
           <t>- Identify CSV/spreadsheet export features that include untrusted input.
 - Verify whether attacker-controlled values are interpreted as formulas when the export is opened in common spreadsheet applications.
@@ -3564,50 +3591,50 @@
 - Assess practical impact based on who opens the export and how it is used.</t>
         </is>
       </c>
-      <c r="E93" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F93" s="18" t="n"/>
-    </row>
-    <row r="94" ht="99" customHeight="1" s="82">
-      <c r="A94" s="19" t="n"/>
-      <c r="B94" s="34" t="inlineStr">
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="n"/>
+    </row>
+    <row r="95" ht="99" customHeight="1" s="82">
+      <c r="A95" s="19" t="n"/>
+      <c r="B95" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-22</t>
         </is>
       </c>
-      <c r="C94" s="15">
+      <c r="C95" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/22-Prototype_Pollution", "Prototype Pollution")</f>
         <v/>
       </c>
-      <c r="D94" s="16" t="inlineStr">
+      <c r="D95" s="16" t="inlineStr">
         <is>
           <t>- Identify functions and libraries that recursively merge, clone, or assign user-controlled properties.
 - Determine whether user input can reach and modify `Object.prototype`.
 - Identify gadgets that turn prototype pollution into a concrete impact.</t>
         </is>
       </c>
-      <c r="E94" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F94" s="18" t="n"/>
-    </row>
-    <row r="95" ht="165" customHeight="1" s="82">
-      <c r="A95" s="19" t="n"/>
-      <c r="B95" s="34" t="inlineStr">
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="n"/>
+    </row>
+    <row r="96" ht="165" customHeight="1" s="82">
+      <c r="A96" s="19" t="n"/>
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>WSTG-INJT-23</t>
         </is>
       </c>
-      <c r="C95" s="15">
+      <c r="C96" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/23-Insecure_Deserialization", "Insecure Deserialization")</f>
         <v/>
       </c>
-      <c r="D95" s="16" t="inlineStr">
+      <c r="D96" s="16" t="inlineStr">
         <is>
           <t>- Identify entry points where the application accepts serialized objects from untrusted
 - urces (for example, HTTP headers, parameters, or cookies).
@@ -3617,174 +3644,150 @@
 - pact.</t>
         </is>
       </c>
-      <c r="E95" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F95" s="18" t="n"/>
-    </row>
-    <row r="96" ht="15" customHeight="1" s="82">
-      <c r="A96" s="97" t="n"/>
-      <c r="B96" s="98" t="n"/>
-      <c r="C96" s="99" t="n"/>
-      <c r="D96" s="99" t="n"/>
-      <c r="E96" s="99" t="n"/>
-      <c r="F96" s="99" t="n"/>
-    </row>
-    <row r="97" ht="47.25" customHeight="1" s="82">
-      <c r="A97" s="9" t="n"/>
-      <c r="B97" s="100" t="inlineStr">
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="n"/>
+    </row>
+    <row r="97" ht="15" customHeight="1" s="82">
+      <c r="A97" s="97" t="n"/>
+      <c r="B97" s="98" t="n"/>
+      <c r="C97" s="99" t="n"/>
+      <c r="D97" s="99" t="n"/>
+      <c r="E97" s="99" t="n"/>
+      <c r="F97" s="99" t="n"/>
+    </row>
+    <row r="98" ht="47.25" customHeight="1" s="82">
+      <c r="A98" s="9" t="n"/>
+      <c r="B98" s="100" t="inlineStr">
         <is>
           <t>Error Handling</t>
         </is>
       </c>
-      <c r="C97" s="101" t="inlineStr">
+      <c r="C98" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D97" s="101" t="inlineStr">
+      <c r="D98" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E97" s="101" t="inlineStr">
+      <c r="E98" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F97" s="101" t="inlineStr">
+      <c r="F98" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="33" customHeight="1" s="82">
-      <c r="A98" s="19" t="n"/>
-      <c r="B98" s="34" t="inlineStr">
+    <row r="99" ht="33" customHeight="1" s="82">
+      <c r="A99" s="19" t="n"/>
+      <c r="B99" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C98" s="15">
+      <c r="C99" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/01-Improper_Error_Handling", "Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D99" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="n"/>
-    </row>
-    <row r="99" ht="16.5" customHeight="1" s="82">
-      <c r="A99" s="19" t="n"/>
-      <c r="B99" s="34" t="inlineStr">
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="n"/>
+    </row>
+    <row r="100" ht="16.5" customHeight="1" s="82">
+      <c r="A100" s="19" t="n"/>
+      <c r="B100" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C99" s="15">
+      <c r="C100" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/02-Stack_Traces", "Stack Traces")</f>
         <v/>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D100" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E99" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F99" s="18" t="n"/>
-    </row>
-    <row r="100" ht="15" customHeight="1" s="82">
-      <c r="A100" s="97" t="n"/>
-      <c r="B100" s="98" t="n"/>
-      <c r="C100" s="99" t="n"/>
-      <c r="D100" s="99" t="n"/>
-      <c r="E100" s="99" t="n"/>
-      <c r="F100" s="99" t="n"/>
-    </row>
-    <row r="101" ht="47.25" customHeight="1" s="82">
-      <c r="A101" s="9" t="n"/>
-      <c r="B101" s="100" t="inlineStr">
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="n"/>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="82">
+      <c r="A101" s="97" t="n"/>
+      <c r="B101" s="98" t="n"/>
+      <c r="C101" s="99" t="n"/>
+      <c r="D101" s="99" t="n"/>
+      <c r="E101" s="99" t="n"/>
+      <c r="F101" s="99" t="n"/>
+    </row>
+    <row r="102" ht="47.25" customHeight="1" s="82">
+      <c r="A102" s="9" t="n"/>
+      <c r="B102" s="100" t="inlineStr">
         <is>
           <t>Weak Cryptography</t>
         </is>
       </c>
-      <c r="C101" s="101" t="inlineStr">
+      <c r="C102" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D101" s="101" t="inlineStr">
+      <c r="D102" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E101" s="101" t="inlineStr">
+      <c r="E102" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F101" s="101" t="inlineStr">
+      <c r="F102" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="82.5" customHeight="1" s="82">
-      <c r="A102" s="19" t="n"/>
-      <c r="B102" s="34" t="inlineStr">
+    <row r="103" ht="82.5" customHeight="1" s="82">
+      <c r="A103" s="19" t="n"/>
+      <c r="B103" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C102" s="15">
+      <c r="C103" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/01-Weak_Transport_Layer_Security", "Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D103" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
-      <c r="E102" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F102" s="18" t="n"/>
-    </row>
-    <row r="103" ht="49.5" customHeight="1" s="82">
-      <c r="A103" s="19" t="n"/>
-      <c r="B103" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-02</t>
-        </is>
-      </c>
-      <c r="C103" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
-        <v/>
-      </c>
-      <c r="D103" s="16" t="inlineStr">
-        <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
-        </is>
-      </c>
       <c r="E103" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3796,146 +3799,170 @@
       <c r="A104" s="19" t="n"/>
       <c r="B104" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C104" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="n"/>
+    </row>
+    <row r="105" ht="49.5" customHeight="1" s="82">
+      <c r="A105" s="19" t="n"/>
+      <c r="B105" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CRYP-03</t>
         </is>
       </c>
-      <c r="C104" s="15">
+      <c r="C105" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/03-Sensitive_Information_Sent_via_Unencrypted_Channels", "Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="D105" s="16" t="inlineStr">
         <is>
           <t>- Identify sensitive information transmitted through the various channels.
 - Assess the privacy and security of the channels used.</t>
         </is>
       </c>
-      <c r="E104" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F104" s="18" t="n"/>
-    </row>
-    <row r="105" ht="33" customHeight="1" s="82">
-      <c r="A105" s="19" t="n"/>
-      <c r="B105" s="34" t="inlineStr">
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="n"/>
+    </row>
+    <row r="106" ht="33" customHeight="1" s="82">
+      <c r="A106" s="19" t="n"/>
+      <c r="B106" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-04</t>
         </is>
       </c>
-      <c r="C105" s="15">
+      <c r="C106" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/04-Weak_Cryptographic_Primitives", "Weak Cryptographic Primitives")</f>
         <v/>
       </c>
-      <c r="D105" s="16" t="inlineStr">
+      <c r="D106" s="16" t="inlineStr">
         <is>
           <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
-      <c r="E105" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F105" s="18" t="n"/>
-    </row>
-    <row r="106" ht="15" customHeight="1" s="82">
-      <c r="A106" s="97" t="n"/>
-      <c r="B106" s="98" t="n"/>
-      <c r="C106" s="99" t="n"/>
-      <c r="D106" s="99" t="n"/>
-      <c r="E106" s="99" t="n"/>
-      <c r="F106" s="99" t="n"/>
-    </row>
-    <row r="107" ht="47.25" customHeight="1" s="82">
-      <c r="A107" s="9" t="n"/>
-      <c r="B107" s="100" t="inlineStr">
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="n"/>
+    </row>
+    <row r="107" ht="15" customHeight="1" s="82">
+      <c r="A107" s="97" t="n"/>
+      <c r="B107" s="98" t="n"/>
+      <c r="C107" s="99" t="n"/>
+      <c r="D107" s="99" t="n"/>
+      <c r="E107" s="99" t="n"/>
+      <c r="F107" s="99" t="n"/>
+    </row>
+    <row r="108" ht="47.25" customHeight="1" s="82">
+      <c r="A108" s="9" t="n"/>
+      <c r="B108" s="100" t="inlineStr">
         <is>
           <t>Business Logic</t>
         </is>
       </c>
-      <c r="C107" s="101" t="inlineStr">
+      <c r="C108" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D107" s="101" t="inlineStr">
+      <c r="D108" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E107" s="101" t="inlineStr">
+      <c r="E108" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F107" s="101" t="inlineStr">
+      <c r="F108" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="82.5" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+    <row r="109" ht="82.5" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C109" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/01-Business_Logic_Data_Validation", "Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="66" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="66" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C110" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/02-Ability_to_Forge_Requests", "Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="148.5" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="n"/>
+    </row>
+    <row r="111" ht="148.5" customHeight="1" s="82">
+      <c r="A111" s="19" t="n"/>
+      <c r="B111" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C111" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/03-Integrity_Checks", "Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D111" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3943,147 +3970,147 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F110" s="18" t="n"/>
-    </row>
-    <row r="111" ht="49.5" customHeight="1" s="82">
-      <c r="A111" s="19" t="n"/>
-      <c r="B111" s="34" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="n"/>
+    </row>
+    <row r="112" ht="49.5" customHeight="1" s="82">
+      <c r="A112" s="19" t="n"/>
+      <c r="B112" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-04</t>
         </is>
       </c>
-      <c r="C111" s="15">
+      <c r="C112" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/04-Process_Timing", "Process Timing")</f>
         <v/>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D112" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for system functionality that may be impacted by time.
 - Develop and execute misuse cases.</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F111" s="18" t="n"/>
-    </row>
-    <row r="112" ht="66" customHeight="1" s="82">
-      <c r="A112" s="19" t="n"/>
-      <c r="B112" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="66" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-05</t>
         </is>
       </c>
-      <c r="C112" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/05-Number_of_Times_a_Function_Can_Be_Used_Limits", "Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Identify functions that must set limits to the times they can be called.
 - Assess if there is a logical limit set on the functions and if it is properly validated.</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="82.5" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="82.5" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-06</t>
         </is>
       </c>
-      <c r="C113" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/06-Circumvention_of_Work_Flows", "Circumvention of Work Flows")</f>
         <v/>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
 - Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="99" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="99" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-07</t>
         </is>
       </c>
-      <c r="C114" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/07-Defenses_Against_Application_Misuse", "Defenses Against Application Misuse")</f>
         <v/>
       </c>
-      <c r="D114" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="99" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="99" customHeight="1" s="82">
+      <c r="A116" s="19" t="n"/>
+      <c r="B116" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C116" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/08-Upload_of_Unexpected_File_Types", "Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="165" customHeight="1" s="82">
-      <c r="A116" s="19" t="n"/>
-      <c r="B116" s="34" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="n"/>
+    </row>
+    <row r="117" ht="165" customHeight="1" s="82">
+      <c r="A117" s="19" t="n"/>
+      <c r="B117" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C116" s="15">
+      <c r="C117" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/09-Upload_of_Malicious_Files", "Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D116" s="16" t="inlineStr">
+      <c r="D117" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4093,114 +4120,91 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F116" s="18" t="n"/>
-    </row>
-    <row r="117" ht="66" customHeight="1" s="82">
-      <c r="A117" s="19" t="n"/>
-      <c r="B117" s="34" t="inlineStr">
+      <c r="E117" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F117" s="18" t="n"/>
+    </row>
+    <row r="118" ht="66" customHeight="1" s="82">
+      <c r="A118" s="19" t="n"/>
+      <c r="B118" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C117" s="15">
+      <c r="C118" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/10-Payment_Functionality", "Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D117" s="16" t="inlineStr">
+      <c r="D118" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E117" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F117" s="18" t="n"/>
-    </row>
-    <row r="118" ht="15" customHeight="1" s="82">
-      <c r="A118" s="97" t="n"/>
-      <c r="B118" s="98" t="n"/>
-      <c r="C118" s="99" t="n"/>
-      <c r="D118" s="99" t="n"/>
-      <c r="E118" s="99" t="n"/>
-      <c r="F118" s="99" t="n"/>
-    </row>
-    <row r="119" ht="47.25" customHeight="1" s="82">
-      <c r="A119" s="9" t="n"/>
-      <c r="B119" s="100" t="inlineStr">
+      <c r="E118" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="n"/>
+    </row>
+    <row r="119" ht="15" customHeight="1" s="82">
+      <c r="A119" s="97" t="n"/>
+      <c r="B119" s="98" t="n"/>
+      <c r="C119" s="99" t="n"/>
+      <c r="D119" s="99" t="n"/>
+      <c r="E119" s="99" t="n"/>
+      <c r="F119" s="99" t="n"/>
+    </row>
+    <row r="120" ht="47.25" customHeight="1" s="82">
+      <c r="A120" s="9" t="n"/>
+      <c r="B120" s="100" t="inlineStr">
         <is>
           <t>Client-side</t>
         </is>
       </c>
-      <c r="C119" s="101" t="inlineStr">
+      <c r="C120" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D119" s="101" t="inlineStr">
+      <c r="D120" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E119" s="101" t="inlineStr">
+      <c r="E120" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F119" s="101" t="inlineStr">
+      <c r="F120" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="33" customHeight="1" s="82">
-      <c r="A120" s="19" t="n"/>
-      <c r="B120" s="34" t="inlineStr">
+    <row r="121" ht="33" customHeight="1" s="82">
+      <c r="A121" s="19" t="n"/>
+      <c r="B121" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-01</t>
         </is>
       </c>
-      <c r="C120" s="15">
+      <c r="C121" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/01-DOM-based_Cross_Site_Scripting", "DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D120" s="16" t="inlineStr">
+      <c r="D121" s="16" t="inlineStr">
         <is>
           <t>- Identify DOM sinks.
 - Build payloads that pertain to every sink type.</t>
         </is>
       </c>
-      <c r="E120" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F120" s="18" t="n"/>
-    </row>
-    <row r="121" ht="16.5" customHeight="1" s="82">
-      <c r="A121" s="19" t="n"/>
-      <c r="B121" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-02</t>
-        </is>
-      </c>
-      <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
-        <v/>
-      </c>
-      <c r="D121" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
-        </is>
-      </c>
       <c r="E121" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4208,20 +4212,20 @@
       </c>
       <c r="F121" s="18" t="n"/>
     </row>
-    <row r="122" ht="33" customHeight="1" s="82">
+    <row r="122" ht="16.5" customHeight="1" s="82">
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-02</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4235,17 +4239,16 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4259,17 +4262,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4283,17 +4286,17 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C125" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
         <v/>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E125" s="18" t="inlineStr">
@@ -4307,42 +4310,43 @@
       <c r="A126" s="19" t="n"/>
       <c r="B126" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-06</t>
+        </is>
+      </c>
+      <c r="C126" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
+        <v/>
+      </c>
+      <c r="D126" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
+        </is>
+      </c>
+      <c r="E126" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F126" s="18" t="n"/>
+    </row>
+    <row r="127" ht="33" customHeight="1" s="82">
+      <c r="A127" s="19" t="n"/>
+      <c r="B127" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-07</t>
         </is>
       </c>
-      <c r="C126" s="15">
+      <c r="C127" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/07-Cross_Origin_Resource_Sharing", "Cross Origin Resource Sharing")</f>
         <v/>
       </c>
-      <c r="D126" s="16" t="inlineStr">
+      <c r="D127" s="16" t="inlineStr">
         <is>
           <t>- Identify endpoints that implement CORS.
 - Ensure that the CORS configuration is secure or harmless.</t>
         </is>
       </c>
-      <c r="E126" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F126" s="18" t="n"/>
-    </row>
-    <row r="127" ht="16.5" customHeight="1" s="82">
-      <c r="A127" s="19" t="n"/>
-      <c r="B127" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-09</t>
-        </is>
-      </c>
-      <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
-        <v/>
-      </c>
-      <c r="D127" s="16" t="inlineStr">
-        <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
-        </is>
-      </c>
       <c r="E127" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4350,21 +4354,20 @@
       </c>
       <c r="F127" s="18" t="n"/>
     </row>
-    <row r="128" ht="49.5" customHeight="1" s="82">
+    <row r="128" ht="16.5" customHeight="1" s="82">
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E128" s="18" t="inlineStr">
@@ -4378,90 +4381,91 @@
       <c r="A129" s="19" t="n"/>
       <c r="B129" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-10</t>
+        </is>
+      </c>
+      <c r="C129" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
+        <v/>
+      </c>
+      <c r="D129" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
+        </is>
+      </c>
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="n"/>
+    </row>
+    <row r="130" ht="49.5" customHeight="1" s="82">
+      <c r="A130" s="19" t="n"/>
+      <c r="B130" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-11</t>
         </is>
       </c>
-      <c r="C129" s="15">
+      <c r="C130" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/11-Web_Messaging", "Web Messaging")</f>
         <v/>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="16" t="inlineStr">
         <is>
           <t>- Assess the security of the message's origin.
 - Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F129" s="18" t="n"/>
-    </row>
-    <row r="130" ht="82.5" customHeight="1" s="82">
-      <c r="A130" s="19" t="n"/>
-      <c r="B130" s="34" t="inlineStr">
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="n"/>
+    </row>
+    <row r="131" ht="82.5" customHeight="1" s="82">
+      <c r="A131" s="19" t="n"/>
+      <c r="B131" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-12</t>
         </is>
       </c>
-      <c r="C130" s="15">
+      <c r="C131" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/12-Browser_Storage", "Browser Storage")</f>
         <v/>
       </c>
-      <c r="D130" s="16" t="inlineStr">
+      <c r="D131" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the site is storing sensitive data in client-side storage.
 - The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F130" s="18" t="n"/>
-    </row>
-    <row r="131" ht="49.5" customHeight="1" s="82">
-      <c r="A131" s="19" t="n"/>
-      <c r="B131" s="34" t="inlineStr">
+      <c r="E131" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F131" s="18" t="n"/>
+    </row>
+    <row r="132" ht="49.5" customHeight="1" s="82">
+      <c r="A132" s="19" t="n"/>
+      <c r="B132" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-13</t>
         </is>
       </c>
-      <c r="C131" s="15">
+      <c r="C132" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/13-Cross_Site_Script_Inclusion", "Cross Site Script Inclusion")</f>
         <v/>
       </c>
-      <c r="D131" s="16" t="inlineStr">
+      <c r="D132" s="16" t="inlineStr">
         <is>
           <t>- Locate sensitive data across the system.
 - Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
-      <c r="E131" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F131" s="18" t="n"/>
-    </row>
-    <row r="132" ht="16.5" customHeight="1" s="82">
-      <c r="A132" s="19" t="n"/>
-      <c r="B132" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D132" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E132" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4469,108 +4473,108 @@
       </c>
       <c r="F132" s="18" t="n"/>
     </row>
-    <row r="133" ht="99" customHeight="1" s="82">
+    <row r="133" ht="16.5" customHeight="1" s="82">
       <c r="A133" s="19" t="n"/>
       <c r="B133" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-14</t>
+        </is>
+      </c>
+      <c r="C133" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
+        <v/>
+      </c>
+      <c r="D133" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="n"/>
+    </row>
+    <row r="134" ht="99" customHeight="1" s="82">
+      <c r="A134" s="19" t="n"/>
+      <c r="B134" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-15</t>
         </is>
       </c>
-      <c r="C133" s="15">
+      <c r="C134" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/15-Client-Side_Template_Injection", "Client-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D133" s="16" t="inlineStr">
+      <c r="D134" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F133" s="18" t="n"/>
-    </row>
-    <row r="134" ht="15" customHeight="1" s="82">
-      <c r="A134" s="97" t="n"/>
-      <c r="B134" s="98" t="n"/>
-      <c r="C134" s="99" t="n"/>
-      <c r="D134" s="99" t="n"/>
-      <c r="E134" s="99" t="n"/>
-      <c r="F134" s="99" t="n"/>
-    </row>
-    <row r="135" ht="47.25" customHeight="1" s="82">
-      <c r="A135" s="9" t="n"/>
-      <c r="B135" s="100" t="inlineStr">
+      <c r="E134" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F134" s="18" t="n"/>
+    </row>
+    <row r="135" ht="15" customHeight="1" s="82">
+      <c r="A135" s="97" t="n"/>
+      <c r="B135" s="98" t="n"/>
+      <c r="C135" s="99" t="n"/>
+      <c r="D135" s="99" t="n"/>
+      <c r="E135" s="99" t="n"/>
+      <c r="F135" s="99" t="n"/>
+    </row>
+    <row r="136" ht="47.25" customHeight="1" s="82">
+      <c r="A136" s="9" t="n"/>
+      <c r="B136" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C135" s="101" t="inlineStr">
+      <c r="C136" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D135" s="101" t="inlineStr">
+      <c r="D136" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E135" s="101" t="inlineStr">
+      <c r="E136" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F135" s="101" t="inlineStr">
+      <c r="F136" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="99" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
+    <row r="137" ht="99" customHeight="1" s="82">
+      <c r="A137" s="19" t="n"/>
+      <c r="B137" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C136" s="15">
+      <c r="C137" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D136" s="16" t="inlineStr">
+      <c r="D137" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E136" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F136" s="18" t="n"/>
-    </row>
-    <row r="137" ht="66" customHeight="1" s="82">
-      <c r="A137" s="19" t="n"/>
-      <c r="B137" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-02</t>
-        </is>
-      </c>
-      <c r="C137" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D137" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
       <c r="E137" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4578,47 +4582,47 @@
       </c>
       <c r="F137" s="18" t="n"/>
     </row>
-    <row r="138" ht="132" customHeight="1" s="82">
+    <row r="138" ht="66" customHeight="1" s="82">
       <c r="A138" s="19" t="n"/>
       <c r="B138" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C138" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D138" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
+      <c r="E138" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F138" s="18" t="n"/>
+    </row>
+    <row r="139" ht="132" customHeight="1" s="82">
+      <c r="A139" s="19" t="n"/>
+      <c r="B139" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C138" s="15">
+      <c r="C139" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Excessive_Data_Exposure", "Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D138" s="16" t="inlineStr">
+      <c r="D139" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E138" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F138" s="18" t="n"/>
-    </row>
-    <row r="139" ht="82.5" customHeight="1" s="82">
-      <c r="A139" s="19" t="n"/>
-      <c r="B139" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-04</t>
-        </is>
-      </c>
-      <c r="C139" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D139" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
       <c r="E139" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4626,38 +4630,61 @@
       </c>
       <c r="F139" s="18" t="n"/>
     </row>
-    <row r="140" ht="66" customHeight="1" s="82">
+    <row r="140" ht="82.5" customHeight="1" s="82">
       <c r="A140" s="19" t="n"/>
       <c r="B140" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C140" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D140" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="66" customHeight="1" s="82">
+      <c r="A141" s="19" t="n"/>
+      <c r="B141" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C140" s="15">
+      <c r="C141" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-GraphQL", "GraphQL")</f>
         <v/>
       </c>
-      <c r="D140" s="16" t="inlineStr">
+      <c r="D141" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="82">
-      <c r="A141" s="97" t="n"/>
-      <c r="B141" s="98" t="n"/>
-      <c r="C141" s="99" t="n"/>
-      <c r="D141" s="99" t="n"/>
-      <c r="E141" s="99" t="n"/>
-      <c r="F141" s="99" t="n"/>
+      <c r="E141" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F141" s="18" t="n"/>
+    </row>
+    <row r="142" ht="15" customHeight="1" s="82">
+      <c r="A142" s="97" t="n"/>
+      <c r="B142" s="98" t="n"/>
+      <c r="C142" s="99" t="n"/>
+      <c r="D142" s="99" t="n"/>
+      <c r="E142" s="99" t="n"/>
+      <c r="F142" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4674,7 +4701,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F141">
+  <conditionalFormatting sqref="B4:F142">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4686,7 +4713,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E99 E100 E103 E104 E105 E106 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-23
Updates based on OWASP/wstg@5ffd31f
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1812,7 +1812,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="82.5" customHeight="1" s="82">
+    <row r="18" ht="165" customHeight="1" s="82">
       <c r="A18" s="19" t="n"/>
       <c r="B18" s="34" t="inlineStr">
         <is>
@@ -1826,7 +1826,8 @@
       <c r="D18" s="16" t="inlineStr">
         <is>
           <t>- Review the applications' configurations set across the network and validate that they are not vulnerable.
-- Validate that used frameworks and systems are secure and not susceptible to known vulnerabilities due to unmaintained software or default settings and credentials.</t>
+- Validate that used frameworks and systems are secure and not susceptible to known vulnerabilities due to unmaintained software or default settings and credentials.
+- Where the infrastructure is cloud-hosted or containerized, review network isolation controls (security groups/NSGs, VPC/subnet layout, load balancer/CDN configuration, service mesh policies, Kubernetes `NetworkPolicy`) for unintended exposure or overly permissive rules.</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -1836,7 +1837,7 @@
       </c>
       <c r="F18" s="18" t="n"/>
     </row>
-    <row r="19" ht="82.5" customHeight="1" s="82">
+    <row r="19" ht="198" customHeight="1" s="82">
       <c r="A19" s="19" t="n"/>
       <c r="B19" s="34" t="inlineStr">
         <is>
@@ -1849,9 +1850,10 @@
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>- Ensure that default and known files have been removed.
-- Validate that no debugging code or extensions are left in the production environments.
-- Review the logging mechanisms set in place for the application.</t>
+          <t>- Ensure that default, sample, and known files have been removed from the deployed platform, container image, or serverless package.
+- Validate that no debugging code, debug endpoints, debug modes, or unused modules/dependencies are left enabled in production environments.
+- Review the logging mechanisms set in place for the application, including what sensitive data may be captured and who/what can access or retain it.
+- Confirm framework-, container-, and serverless-specific production hardening settings are applied rather than left at insecure defaults.</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
@@ -1861,7 +1863,7 @@
       </c>
       <c r="F19" s="18" t="n"/>
     </row>
-    <row r="20" ht="66" customHeight="1" s="82">
+    <row r="20" ht="33" customHeight="1" s="82">
       <c r="A20" s="19" t="n"/>
       <c r="B20" s="34" t="inlineStr">
         <is>
@@ -1874,8 +1876,7 @@
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>- Enumerate sensitive file extensions that might contain raw data such as scripts or credentials
-- Validate that no system framework bypasses exist for the rules that have been set</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -1885,7 +1886,7 @@
       </c>
       <c r="F20" s="18" t="n"/>
     </row>
-    <row r="21" ht="33" customHeight="1" s="82">
+    <row r="21" ht="115.5" customHeight="1" s="82">
       <c r="A21" s="19" t="n"/>
       <c r="B21" s="34" t="inlineStr">
         <is>
@@ -1898,7 +1899,8 @@
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>- Find and analyse unreferenced files that might contain sensitive information.</t>
+          <t>- Find and analyze old, backup, and unreferenced files - including files exposed only through their extension, and objects left in cloud storage - that might contain sensitive information.
+- Validate that no system or framework bypasses exist for any rules put in place to prevent these files from being served.</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -1908,7 +1910,7 @@
       </c>
       <c r="F21" s="18" t="n"/>
     </row>
-    <row r="22" ht="33" customHeight="1" s="82">
+    <row r="22" ht="99" customHeight="1" s="82">
       <c r="A22" s="19" t="n"/>
       <c r="B22" s="34" t="inlineStr">
         <is>
@@ -1921,7 +1923,8 @@
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>- Identify hidden administrator interfaces and functionality.</t>
+          <t>- Identify hidden administrator interfaces and functionality, including cloud, container-orchestration, API-management, and CI/CD management consoles.
+- Check any discovered interface for default, weak, or reused credentials, and for exposure to networks/users beyond those intended.</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -1956,7 +1959,7 @@
       </c>
       <c r="F23" s="18" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="82">
+    <row r="24" ht="132" customHeight="1" s="82">
       <c r="A24" s="19" t="n"/>
       <c r="B24" s="34" t="inlineStr">
         <is>
@@ -1969,7 +1972,9 @@
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>- Review the HSTS header and its validity.</t>
+          <t>- Review the HSTS header, its directives, and their values for consistency with current best practice.
+- Confirm the site is protected against the first-request trust gap, either via preload or an otherwise hardened HTTP-to-HTTPS path.
+- Confirm HSTS is applied consistently across the domain and relevant subdomains, and does not mask mixed-content issues.</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
@@ -1979,7 +1984,7 @@
       </c>
       <c r="F24" s="18" t="n"/>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="82">
+    <row r="25" ht="165" customHeight="1" s="82">
       <c r="A25" s="19" t="n"/>
       <c r="B25" s="34" t="inlineStr">
         <is>
@@ -1987,12 +1992,14 @@
         </is>
       </c>
       <c r="C25" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permission", "File Permission")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permissions", "File Permissions")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>- Review and identify any rogue file permissions.</t>
+          <t>- Review and identify any rogue file permissions on the host filesystem, in container images/filesystems, and on cloud storage objects.
+- Assess whether Kubernetes volume mounts and `securityContext` settings enforce least-privilege access to files and secrets.
+- Identify secrets stored with overly broad permissions, wherever they are held (filesystem, container image, orchestration secret store, cloud secrets manager export, CI artifacts).</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -2002,7 +2009,7 @@
       </c>
       <c r="F25" s="18" t="n"/>
     </row>
-    <row r="26" ht="33" customHeight="1" s="82">
+    <row r="26" ht="148.5" customHeight="1" s="82">
       <c r="A26" s="19" t="n"/>
       <c r="B26" s="34" t="inlineStr">
         <is>
@@ -2015,8 +2022,9 @@
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>- Enumerate all possible domains (previous and current).
-- Identify any forgotten or misconfigured domains.</t>
+          <t>- Enumerate all possible domains (previous and current), including wildcard-covered names.
+- Identify any forgotten or misconfigured domains, and any dangling-service signature not covered by a known response fingerprint.
+- Where a takeover is confirmed feasible, assess whether the parent application's cookies, CORS policy, OAuth redirect validation, or CSP allowlist extend trust to the claimed subdomain.</t>
         </is>
       </c>
       <c r="E26" s="18" t="inlineStr">
@@ -2026,7 +2034,7 @@
       </c>
       <c r="F26" s="18" t="n"/>
     </row>
-    <row r="27" ht="33" customHeight="1" s="82">
+    <row r="27" ht="132" customHeight="1" s="82">
       <c r="A27" s="19" t="n"/>
       <c r="B27" s="34" t="inlineStr">
         <is>
@@ -2039,7 +2047,9 @@
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>- Assess that the access control configuration for the storage services is properly in place.</t>
+          <t>- Assess that the access control configuration for the storage services (bucket/container-level public access, and object/principal-level ACLs or IAM policies) is properly in place.
+- Assess whether signed/presigned URLs are scoped, time-limited, and handled appropriately.
+- Assess whether object versioning and lifecycle configuration could expose old or supposedly-removed sensitive data.</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
@@ -2072,7 +2082,7 @@
       </c>
       <c r="F28" s="18" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="82">
+    <row r="29" ht="115.5" customHeight="1" s="82">
       <c r="A29" s="19" t="n"/>
       <c r="B29" s="34" t="inlineStr">
         <is>
@@ -2085,7 +2095,8 @@
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>- Make sure application paths are configured correctly.</t>
+          <t>- Make sure application paths are configured and normalized consistently across all components (application, proxy, cache, CDN, WAF) that make decisions based on the path.
+- Identify cases where trailing slashes, case sensitivity, or encoding differences cause a security control (auth/access rules, routing, cache keying) to be bypassed or behave inconsistently.</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-23 (#1542)
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1812,7 +1812,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="82.5" customHeight="1" s="82">
+    <row r="18" ht="165" customHeight="1" s="82">
       <c r="A18" s="19" t="n"/>
       <c r="B18" s="34" t="inlineStr">
         <is>
@@ -1826,7 +1826,8 @@
       <c r="D18" s="16" t="inlineStr">
         <is>
           <t>- Review the applications' configurations set across the network and validate that they are not vulnerable.
-- Validate that used frameworks and systems are secure and not susceptible to known vulnerabilities due to unmaintained software or default settings and credentials.</t>
+- Validate that used frameworks and systems are secure and not susceptible to known vulnerabilities due to unmaintained software or default settings and credentials.
+- Where the infrastructure is cloud-hosted or containerized, review network isolation controls (security groups/NSGs, VPC/subnet layout, load balancer/CDN configuration, service mesh policies, Kubernetes `NetworkPolicy`) for unintended exposure or overly permissive rules.</t>
         </is>
       </c>
       <c r="E18" s="18" t="inlineStr">
@@ -1836,7 +1837,7 @@
       </c>
       <c r="F18" s="18" t="n"/>
     </row>
-    <row r="19" ht="82.5" customHeight="1" s="82">
+    <row r="19" ht="198" customHeight="1" s="82">
       <c r="A19" s="19" t="n"/>
       <c r="B19" s="34" t="inlineStr">
         <is>
@@ -1849,9 +1850,10 @@
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>- Ensure that default and known files have been removed.
-- Validate that no debugging code or extensions are left in the production environments.
-- Review the logging mechanisms set in place for the application.</t>
+          <t>- Ensure that default, sample, and known files have been removed from the deployed platform, container image, or serverless package.
+- Validate that no debugging code, debug endpoints, debug modes, or unused modules/dependencies are left enabled in production environments.
+- Review the logging mechanisms set in place for the application, including what sensitive data may be captured and who/what can access or retain it.
+- Confirm framework-, container-, and serverless-specific production hardening settings are applied rather than left at insecure defaults.</t>
         </is>
       </c>
       <c r="E19" s="18" t="inlineStr">
@@ -1861,7 +1863,7 @@
       </c>
       <c r="F19" s="18" t="n"/>
     </row>
-    <row r="20" ht="66" customHeight="1" s="82">
+    <row r="20" ht="33" customHeight="1" s="82">
       <c r="A20" s="19" t="n"/>
       <c r="B20" s="34" t="inlineStr">
         <is>
@@ -1874,8 +1876,7 @@
       </c>
       <c r="D20" s="16" t="inlineStr">
         <is>
-          <t>- Enumerate sensitive file extensions that might contain raw data such as scripts or credentials
-- Validate that no system framework bypasses exist for the rules that have been set</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -1885,7 +1886,7 @@
       </c>
       <c r="F20" s="18" t="n"/>
     </row>
-    <row r="21" ht="33" customHeight="1" s="82">
+    <row r="21" ht="115.5" customHeight="1" s="82">
       <c r="A21" s="19" t="n"/>
       <c r="B21" s="34" t="inlineStr">
         <is>
@@ -1898,7 +1899,8 @@
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>- Find and analyse unreferenced files that might contain sensitive information.</t>
+          <t>- Find and analyze old, backup, and unreferenced files - including files exposed only through their extension, and objects left in cloud storage - that might contain sensitive information.
+- Validate that no system or framework bypasses exist for any rules put in place to prevent these files from being served.</t>
         </is>
       </c>
       <c r="E21" s="18" t="inlineStr">
@@ -1908,7 +1910,7 @@
       </c>
       <c r="F21" s="18" t="n"/>
     </row>
-    <row r="22" ht="33" customHeight="1" s="82">
+    <row r="22" ht="99" customHeight="1" s="82">
       <c r="A22" s="19" t="n"/>
       <c r="B22" s="34" t="inlineStr">
         <is>
@@ -1921,7 +1923,8 @@
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>- Identify hidden administrator interfaces and functionality.</t>
+          <t>- Identify hidden administrator interfaces and functionality, including cloud, container-orchestration, API-management, and CI/CD management consoles.
+- Check any discovered interface for default, weak, or reused credentials, and for exposure to networks/users beyond those intended.</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
@@ -1956,7 +1959,7 @@
       </c>
       <c r="F23" s="18" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="82">
+    <row r="24" ht="132" customHeight="1" s="82">
       <c r="A24" s="19" t="n"/>
       <c r="B24" s="34" t="inlineStr">
         <is>
@@ -1969,7 +1972,9 @@
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>- Review the HSTS header and its validity.</t>
+          <t>- Review the HSTS header, its directives, and their values for consistency with current best practice.
+- Confirm the site is protected against the first-request trust gap, either via preload or an otherwise hardened HTTP-to-HTTPS path.
+- Confirm HSTS is applied consistently across the domain and relevant subdomains, and does not mask mixed-content issues.</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
@@ -1979,7 +1984,7 @@
       </c>
       <c r="F24" s="18" t="n"/>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="82">
+    <row r="25" ht="165" customHeight="1" s="82">
       <c r="A25" s="19" t="n"/>
       <c r="B25" s="34" t="inlineStr">
         <is>
@@ -1987,12 +1992,14 @@
         </is>
       </c>
       <c r="C25" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permission", "File Permission")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permissions", "File Permissions")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>- Review and identify any rogue file permissions.</t>
+          <t>- Review and identify any rogue file permissions on the host filesystem, in container images/filesystems, and on cloud storage objects.
+- Assess whether Kubernetes volume mounts and `securityContext` settings enforce least-privilege access to files and secrets.
+- Identify secrets stored with overly broad permissions, wherever they are held (filesystem, container image, orchestration secret store, cloud secrets manager export, CI artifacts).</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -2002,7 +2009,7 @@
       </c>
       <c r="F25" s="18" t="n"/>
     </row>
-    <row r="26" ht="33" customHeight="1" s="82">
+    <row r="26" ht="148.5" customHeight="1" s="82">
       <c r="A26" s="19" t="n"/>
       <c r="B26" s="34" t="inlineStr">
         <is>
@@ -2015,8 +2022,9 @@
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>- Enumerate all possible domains (previous and current).
-- Identify any forgotten or misconfigured domains.</t>
+          <t>- Enumerate all possible domains (previous and current), including wildcard-covered names.
+- Identify any forgotten or misconfigured domains, and any dangling-service signature not covered by a known response fingerprint.
+- Where a takeover is confirmed feasible, assess whether the parent application's cookies, CORS policy, OAuth redirect validation, or CSP allowlist extend trust to the claimed subdomain.</t>
         </is>
       </c>
       <c r="E26" s="18" t="inlineStr">
@@ -2026,7 +2034,7 @@
       </c>
       <c r="F26" s="18" t="n"/>
     </row>
-    <row r="27" ht="33" customHeight="1" s="82">
+    <row r="27" ht="132" customHeight="1" s="82">
       <c r="A27" s="19" t="n"/>
       <c r="B27" s="34" t="inlineStr">
         <is>
@@ -2039,7 +2047,9 @@
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>- Assess that the access control configuration for the storage services is properly in place.</t>
+          <t>- Assess that the access control configuration for the storage services (bucket/container-level public access, and object/principal-level ACLs or IAM policies) is properly in place.
+- Assess whether signed/presigned URLs are scoped, time-limited, and handled appropriately.
+- Assess whether object versioning and lifecycle configuration could expose old or supposedly-removed sensitive data.</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
@@ -2072,7 +2082,7 @@
       </c>
       <c r="F28" s="18" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="82">
+    <row r="29" ht="115.5" customHeight="1" s="82">
       <c r="A29" s="19" t="n"/>
       <c r="B29" s="34" t="inlineStr">
         <is>
@@ -2085,7 +2095,8 @@
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>- Make sure application paths are configured correctly.</t>
+          <t>- Make sure application paths are configured and normalized consistently across all components (application, proxy, cache, CDN, WAF) that make decisions based on the path.
+- Identify cases where trailing slashes, case sensitivity, or encoding differences cause a security control (auth/access rules, routing, cache keying) to be bypassed or behave inconsistently.</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-10-14
Updates based on OWASP/wstg@165ae5c
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -3913,7 +3913,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="82.5" customHeight="1" s="82">
+    <row r="109" ht="132" customHeight="1" s="82">
       <c r="A109" s="19" t="n"/>
       <c r="B109" s="34" t="inlineStr">
         <is>
@@ -3928,7 +3928,8 @@
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
-- Attempt to break the format of the expected data and analyze how the application is handling it.</t>
+- Attempt to break the format of the expected data and analyze how the application is handling it.
+- Determine whether parameters that the frontend restricts (type, range, set of allowed values, or relationship to other fields) are restricted again on the server.</t>
         </is>
       </c>
       <c r="E109" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-10-15
Updates based on OWASP/wstg@b69d0c0
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -4697,6 +4697,68 @@
       <c r="D142" s="99" t="n"/>
       <c r="E142" s="99" t="n"/>
       <c r="F142" s="99" t="n"/>
+    </row>
+    <row r="143" ht="47.25" customHeight="1" s="82">
+      <c r="A143" s="9" t="n"/>
+      <c r="B143" s="100" t="inlineStr">
+        <is>
+          <t>WebAssembly Testing</t>
+        </is>
+      </c>
+      <c r="C143" s="101" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="D143" s="101" t="inlineStr">
+        <is>
+          <t>Objectives</t>
+        </is>
+      </c>
+      <c r="E143" s="101" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F143" s="101" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="198" customHeight="1" s="82">
+      <c r="A144" s="19" t="n"/>
+      <c r="B144" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-WASM-01</t>
+        </is>
+      </c>
+      <c r="C144" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/13-WebAssembly_Testing/01-WebAssembly_Reconnaissance", "WebAssembly Reconnaissance")</f>
+        <v/>
+      </c>
+      <c r="D144" s="16" t="inlineStr">
+        <is>
+          <t>- Find all WebAssembly modules loaded by the target application, including those not named `.wasm`, compressed, lazy-loaded, loaded through `fetch`, and manual instantiation, or embedded in JavaScript.
+- Identify the compiler toolchain and source language (e.g., C/C++, Rust, Go, .NET) from section metadata, imports, exports, and glue code.
+- Detect exposed debugging artifacts: source maps, DWARF information, and the `name` custom section.
+- Map the infrastructure attack surface by extracting embedded URLs, API endpoints, and internal hostnames or IP addresses.</t>
+        </is>
+      </c>
+      <c r="E144" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F144" s="18" t="n"/>
+    </row>
+    <row r="145" ht="15" customHeight="1" s="82">
+      <c r="A145" s="97" t="n"/>
+      <c r="B145" s="98" t="n"/>
+      <c r="C145" s="99" t="n"/>
+      <c r="D145" s="99" t="n"/>
+      <c r="E145" s="99" t="n"/>
+      <c r="F145" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4713,7 +4775,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F142">
+  <conditionalFormatting sqref="B4:F145">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4725,7 +4787,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E99 E100 E103 E104 E105 E106 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E99 E100 E103 E104 E105 E106 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141 E144" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-10-30
Updates based on OWASP/wstg@ae48eb3
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -3698,7 +3698,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="33" customHeight="1" s="82">
+    <row r="99" ht="66" customHeight="1" s="82">
       <c r="A99" s="19" t="n"/>
       <c r="B99" s="34" t="inlineStr">
         <is>
@@ -3712,7 +3712,8 @@
       <c r="D99" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
-- Analyze the different output returned.</t>
+- Analyze the different output returned.
+- Determine whether errors expose sensitive information or cause the application to fail open.</t>
         </is>
       </c>
       <c r="E99" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-10-30 (#1585)
Updates based on OWASP/wstg@ae48eb3
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -3698,7 +3698,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="33" customHeight="1" s="82">
+    <row r="99" ht="66" customHeight="1" s="82">
       <c r="A99" s="19" t="n"/>
       <c r="B99" s="34" t="inlineStr">
         <is>
@@ -3712,7 +3712,8 @@
       <c r="D99" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
-- Analyze the different output returned.</t>
+- Analyze the different output returned.
+- Determine whether errors expose sensitive information or cause the application to fail open.</t>
         </is>
       </c>
       <c r="E99" s="18" t="inlineStr">

</xml_diff>